<commit_message>
Atualiza painel (08/10/2026 14:49)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD42B021-41C4-4B06-B1F6-F46CE1B5DBFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E3F991B-0B47-4AC2-8ED2-4C31F26C7C7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
   <sheets>
     <sheet name="Captações" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="62">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -92,24 +92,6 @@
     <t>Faixa</t>
   </si>
   <si>
-    <t>Até R$ 300 mil</t>
-  </si>
-  <si>
-    <t>R$ 300 mil a R$ 500 mil</t>
-  </si>
-  <si>
-    <t>R$ 500 mil a R$ 800 mil</t>
-  </si>
-  <si>
-    <t>R$ 800 mil a R$ 1,2 milhão</t>
-  </si>
-  <si>
-    <t>R$ 1,2 milhão a R$ 2 milhões</t>
-  </si>
-  <si>
-    <t>Acima de R$ 2 milhões</t>
-  </si>
-  <si>
     <t>Como funciona: cada imóvel recebe os pontos da faixa em que o seu valor se encaixa (Valor mínimo &lt;= valor &lt;= Valor máximo).</t>
   </si>
   <si>
@@ -227,7 +209,34 @@
     <t>690531104-966</t>
   </si>
   <si>
-    <t>Venda - Com financiamento</t>
+    <t>VENDA - Até R$ 500 mil - sem financiamento</t>
+  </si>
+  <si>
+    <t>VENDA - Até R$ 500 mil - com financiamento</t>
+  </si>
+  <si>
+    <t>VENDA - A partir de R$ 500 mil - sem financiamento</t>
+  </si>
+  <si>
+    <t>VENDA - A partir de R$ 500 mil - com financiamento</t>
+  </si>
+  <si>
+    <t>VENDA - Renovação da Representação</t>
+  </si>
+  <si>
+    <t>VENDA - Cancelamento da Representação</t>
+  </si>
+  <si>
+    <t>VENDA - Se a gestão conquistada for vendida no período da campanha</t>
+  </si>
+  <si>
+    <t>LOCAÇÃO - De R$ 1.200,00 a R$ 2.000,00</t>
+  </si>
+  <si>
+    <t>LOCAÇÃO - A partir de R$ 2.000,00</t>
+  </si>
+  <si>
+    <t>LOCAÇÃO - Cancelamento da captação de locação</t>
   </si>
 </sst>
 </file>
@@ -293,7 +302,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -306,8 +315,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -315,12 +330,36 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -340,6 +379,10 @@
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
@@ -404,8 +447,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BE296B9A-7FB2-47EF-91CE-D94B7341102A}" name="tbFaixas" displayName="tbFaixas" ref="A1:D7" totalsRowShown="0">
-  <autoFilter ref="A1:D7" xr:uid="{BE296B9A-7FB2-47EF-91CE-D94B7341102A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BE296B9A-7FB2-47EF-91CE-D94B7341102A}" name="tbFaixas" displayName="tbFaixas" ref="A1:D11" totalsRowShown="0">
+  <autoFilter ref="A1:D11" xr:uid="{BE296B9A-7FB2-47EF-91CE-D94B7341102A}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{D2501A27-5A99-4009-8294-2BFD28385B1D}" name="Valor mínimo" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{488F6EEF-997C-45E1-B6E8-ADC37F785D66}" name="Valor máximo" dataDxfId="0"/>
@@ -724,57 +767,57 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="C8" s="10">
         <v>4400</v>
@@ -786,42 +829,30 @@
         <v>35</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="C9" s="8">
-        <v>650000</v>
-      </c>
-      <c r="D9" s="9">
-        <v>46302</v>
-      </c>
-      <c r="E9" s="7">
-        <v>180</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C12" s="10">
         <v>4400</v>
@@ -833,87 +864,87 @@
         <v>35</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" s="7" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" s="7" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -928,12 +959,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CFA2527-A1B4-4C70-9FD6-48BF94DAE799}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="18.77734375" customWidth="1"/>
     <col min="3" max="3" width="10.77734375" customWidth="1"/>
-    <col min="4" max="4" width="32.77734375" customWidth="1"/>
+    <col min="4" max="4" width="59.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -951,95 +982,125 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="6">
-        <v>0</v>
-      </c>
-      <c r="B2" s="6">
-        <v>300000</v>
-      </c>
-      <c r="C2">
-        <v>10</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="A2" s="6"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="11">
+        <v>100</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="6"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="13">
+        <v>130</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="11">
+        <v>120</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="6"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="13">
+        <v>150</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="6"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="11">
+        <v>50</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="6"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="13">
+        <v>-50</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="11">
+        <v>200</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="13">
+        <v>50</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="11">
+        <v>70</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="13">
+        <v>-50</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="6">
-        <v>300000.01</v>
-      </c>
-      <c r="B3" s="6">
-        <v>500000</v>
-      </c>
-      <c r="C3">
-        <v>20</v>
-      </c>
-      <c r="D3" t="s">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" s="5" t="s">
         <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="6">
-        <v>500000.01</v>
-      </c>
-      <c r="B4" s="6">
-        <v>800000</v>
-      </c>
-      <c r="C4">
-        <v>30</v>
-      </c>
-      <c r="D4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="6">
-        <v>800000.01</v>
-      </c>
-      <c r="B5" s="6">
-        <v>1200000</v>
-      </c>
-      <c r="C5">
-        <v>45</v>
-      </c>
-      <c r="D5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="6">
-        <v>1200000.01</v>
-      </c>
-      <c r="B6" s="6">
-        <v>2000000</v>
-      </c>
-      <c r="C6">
-        <v>65</v>
-      </c>
-      <c r="D6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="6">
-        <v>2000000.01</v>
-      </c>
-      <c r="B7" s="6"/>
-      <c r="C7">
-        <v>100</v>
-      </c>
-      <c r="D7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
-        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1070,7 +1131,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -1094,7 +1155,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualiza painel (08/10/2026 23:45)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E3F991B-0B47-4AC2-8ED2-4C31F26C7C7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73F8F8D3-0DB8-4B2D-AFB9-E658A0E39F04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
   <sheets>
     <sheet name="Captações" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="69">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -203,9 +203,6 @@
     <t>Locação - Parceria</t>
   </si>
   <si>
-    <t>Locação  - Parceria</t>
-  </si>
-  <si>
     <t>690531104-966</t>
   </si>
   <si>
@@ -237,6 +234,34 @@
   </si>
   <si>
     <t>LOCAÇÃO - Cancelamento da captação de locação</t>
+  </si>
+  <si>
+    <t>690531104-966
+690531057-138</t>
+  </si>
+  <si>
+    <t>Locação  - Parceria
+Venda</t>
+  </si>
+  <si>
+    <t>R$ 4.400,00
+350.000,00</t>
+  </si>
+  <si>
+    <t>07/10/2026
+08/10/2026</t>
+  </si>
+  <si>
+    <t>Locação</t>
+  </si>
+  <si>
+    <t>690701036-76</t>
+  </si>
+  <si>
+    <t>690531008-310</t>
+  </si>
+  <si>
+    <t>Venda - Parceria</t>
   </si>
 </sst>
 </file>
@@ -359,7 +384,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -367,22 +392,31 @@
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
@@ -390,32 +424,32 @@
   </cellStyles>
   <dxfs count="9">
     <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #.##000"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #.##000"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #.##000"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -431,7 +465,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E53" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E53" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
   <autoFilter ref="A1:E53" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F68D7E3E-8D02-41D7-8907-35C934E19501}" name="Corretor" dataDxfId="6"/>
@@ -450,8 +484,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BE296B9A-7FB2-47EF-91CE-D94B7341102A}" name="tbFaixas" displayName="tbFaixas" ref="A1:D11" totalsRowShown="0">
   <autoFilter ref="A1:D11" xr:uid="{BE296B9A-7FB2-47EF-91CE-D94B7341102A}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{D2501A27-5A99-4009-8294-2BFD28385B1D}" name="Valor mínimo" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{488F6EEF-997C-45E1-B6E8-ADC37F785D66}" name="Valor máximo" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{D2501A27-5A99-4009-8294-2BFD28385B1D}" name="Valor mínimo" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{488F6EEF-997C-45E1-B6E8-ADC37F785D66}" name="Valor máximo" dataDxfId="7"/>
     <tableColumn id="3" xr3:uid="{830BDE7B-EA8B-4E6F-A7D4-9A97F158AED2}" name="Pontos"/>
     <tableColumn id="4" xr3:uid="{8056E5D0-FC15-43C2-A6CB-667290BADF20}" name="Faixa"/>
   </tableColumns>
@@ -460,9 +494,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -500,7 +534,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -606,7 +640,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -748,7 +782,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -759,191 +793,230 @@
   <dimension ref="A1:F28"/>
   <sheetFormatPr defaultColWidth="26.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="26.44140625" style="7"/>
-    <col min="3" max="3" width="26.44140625" style="8"/>
-    <col min="4" max="4" width="26.44140625" style="9"/>
-    <col min="5" max="16384" width="26.44140625" style="7"/>
+    <col min="1" max="2" width="26.44140625" style="11"/>
+    <col min="3" max="3" width="26.44140625" style="12"/>
+    <col min="4" max="4" width="26.44140625" style="13"/>
+    <col min="5" max="16384" width="26.44140625" style="11"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="11" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="11" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="11" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="11" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="11" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="11" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
+      <c r="B7" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="C7" s="14">
+        <v>1350000</v>
+      </c>
+      <c r="D7" s="13">
+        <v>46303</v>
+      </c>
+      <c r="E7" s="11">
+        <v>75</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="E8" s="15">
+        <v>135</v>
+      </c>
+      <c r="F8" s="15" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C10" s="14">
+        <v>2190</v>
+      </c>
+      <c r="D10" s="13">
+        <v>46302</v>
+      </c>
+      <c r="E10" s="11">
+        <v>70</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="11" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" s="14">
+        <v>4400</v>
+      </c>
+      <c r="D12" s="13">
+        <v>46302</v>
+      </c>
+      <c r="E12" s="11">
+        <v>35</v>
+      </c>
+      <c r="F12" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="C8" s="10">
-        <v>4400</v>
-      </c>
-      <c r="D8" s="9">
-        <v>46302</v>
-      </c>
-      <c r="E8" s="7">
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="E15" s="11">
+        <v>75</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" s="11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" s="11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="F8" s="7" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="7" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="C12" s="10">
-        <v>4400</v>
-      </c>
-      <c r="D12" s="9">
-        <v>46302</v>
-      </c>
-      <c r="E12" s="7">
-        <v>35</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="7" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" s="7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" s="7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A19" s="7" t="s">
-        <v>35</v>
-      </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="11" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="11" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A22" s="7" t="s">
+      <c r="A22" s="11" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A23" s="7" t="s">
+      <c r="A23" s="11" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A24" s="7" t="s">
+      <c r="A24" s="11" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A25" s="7" t="s">
+      <c r="A25" s="11" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A26" s="7" t="s">
+      <c r="A26" s="11" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A27" s="7" t="s">
+      <c r="A27" s="11" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A28" s="7" t="s">
+      <c r="A28" s="11" t="s">
         <v>46</v>
       </c>
     </row>
@@ -984,101 +1057,101 @@
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="6"/>
       <c r="B2" s="6"/>
-      <c r="C2" s="11">
+      <c r="C2" s="7">
         <v>100</v>
       </c>
-      <c r="D2" s="12" t="s">
-        <v>52</v>
+      <c r="D2" s="8" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="6"/>
       <c r="B3" s="6"/>
-      <c r="C3" s="13">
+      <c r="C3" s="9">
         <v>130</v>
       </c>
-      <c r="D3" s="14" t="s">
-        <v>53</v>
+      <c r="D3" s="10" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="6"/>
       <c r="B4" s="6"/>
-      <c r="C4" s="11">
+      <c r="C4" s="7">
         <v>120</v>
       </c>
-      <c r="D4" s="12" t="s">
-        <v>54</v>
+      <c r="D4" s="8" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="6"/>
       <c r="B5" s="6"/>
-      <c r="C5" s="13">
+      <c r="C5" s="9">
         <v>150</v>
       </c>
-      <c r="D5" s="14" t="s">
-        <v>55</v>
+      <c r="D5" s="10" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="6"/>
       <c r="B6" s="6"/>
-      <c r="C6" s="11">
+      <c r="C6" s="7">
         <v>50</v>
       </c>
-      <c r="D6" s="12" t="s">
-        <v>56</v>
+      <c r="D6" s="8" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="6"/>
       <c r="B7" s="6"/>
-      <c r="C7" s="13">
+      <c r="C7" s="9">
         <v>-50</v>
       </c>
-      <c r="D7" s="14" t="s">
-        <v>57</v>
+      <c r="D7" s="10" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="6"/>
       <c r="B8" s="6"/>
-      <c r="C8" s="11">
+      <c r="C8" s="7">
         <v>200</v>
       </c>
-      <c r="D8" s="12" t="s">
-        <v>58</v>
+      <c r="D8" s="8" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
-      <c r="C9" s="13">
+      <c r="C9" s="9">
         <v>50</v>
       </c>
-      <c r="D9" s="14" t="s">
-        <v>59</v>
+      <c r="D9" s="10" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="6"/>
       <c r="B10" s="6"/>
-      <c r="C10" s="11">
+      <c r="C10" s="7">
         <v>70</v>
       </c>
-      <c r="D10" s="12" t="s">
-        <v>60</v>
+      <c r="D10" s="8" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="6"/>
       <c r="B11" s="6"/>
-      <c r="C11" s="13">
+      <c r="C11" s="9">
         <v>-50</v>
       </c>
-      <c r="D11" s="14" t="s">
-        <v>61</v>
+      <c r="D11" s="10" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualiza painel (09/10/2026 00:05)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73F8F8D3-0DB8-4B2D-AFB9-E658A0E39F04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46AD5009-AA9C-45F4-B7B6-77B91BE9288E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="71">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -262,6 +262,12 @@
   </si>
   <si>
     <t>Venda - Parceria</t>
+  </si>
+  <si>
+    <t>Diego</t>
+  </si>
+  <si>
+    <t>Casa - condomínio</t>
   </si>
 </sst>
 </file>
@@ -424,10 +430,10 @@
   </cellStyles>
   <dxfs count="9">
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #.##000"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #.##000"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -446,10 +452,10 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #.##000"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #.##000"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -465,7 +471,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E53" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E53" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
   <autoFilter ref="A1:E53" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F68D7E3E-8D02-41D7-8907-35C934E19501}" name="Corretor" dataDxfId="6"/>
@@ -484,8 +490,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BE296B9A-7FB2-47EF-91CE-D94B7341102A}" name="tbFaixas" displayName="tbFaixas" ref="A1:D11" totalsRowShown="0">
   <autoFilter ref="A1:D11" xr:uid="{BE296B9A-7FB2-47EF-91CE-D94B7341102A}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{D2501A27-5A99-4009-8294-2BFD28385B1D}" name="Valor mínimo" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{488F6EEF-997C-45E1-B6E8-ADC37F785D66}" name="Valor máximo" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{D2501A27-5A99-4009-8294-2BFD28385B1D}" name="Valor mínimo" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{488F6EEF-997C-45E1-B6E8-ADC37F785D66}" name="Valor máximo" dataDxfId="0"/>
     <tableColumn id="3" xr3:uid="{830BDE7B-EA8B-4E6F-A7D4-9A97F158AED2}" name="Pontos"/>
     <tableColumn id="4" xr3:uid="{8056E5D0-FC15-43C2-A6CB-667290BADF20}" name="Faixa"/>
   </tableColumns>
@@ -494,9 +500,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -534,7 +540,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -640,7 +646,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -782,7 +788,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -790,7 +796,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51DF420C-6417-4C8E-9CA8-EAE7781FF48D}">
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr defaultColWidth="26.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="26.44140625" style="11"/>
@@ -960,64 +966,75 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="11" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
         <v>46</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B29" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="E29" s="11">
+        <v>190</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza painel (09/10/2026 05:16)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46AD5009-AA9C-45F4-B7B6-77B91BE9288E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44A3A33C-32F6-4220-85DF-5CCD6AD835E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -1033,6 +1033,12 @@
       <c r="B29" s="11" t="s">
         <v>70</v>
       </c>
+      <c r="C29" s="14">
+        <v>1350000</v>
+      </c>
+      <c r="D29" s="13">
+        <v>46303</v>
+      </c>
       <c r="E29" s="11">
         <v>190</v>
       </c>

</xml_diff>

<commit_message>
Atualiza painel (09/10/2026 05:28)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44A3A33C-32F6-4220-85DF-5CCD6AD835E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BDDC497-46D4-4479-8B58-499138923FF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="69">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -262,12 +262,6 @@
   </si>
   <si>
     <t>Venda - Parceria</t>
-  </si>
-  <si>
-    <t>Diego</t>
-  </si>
-  <si>
-    <t>Casa - condomínio</t>
   </si>
 </sst>
 </file>
@@ -966,82 +960,68 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="11" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A29" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="B29" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="C29" s="14">
-        <v>1350000</v>
-      </c>
-      <c r="D29" s="13">
-        <v>46303</v>
-      </c>
-      <c r="E29" s="11">
-        <v>190</v>
-      </c>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C29" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>

<commit_message>
Atualiza painel (09/10/2026 16:14)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BDDC497-46D4-4479-8B58-499138923FF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B97875DA-4664-46F2-8FBB-A3A4A3AB644A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="70">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -262,6 +262,9 @@
   </si>
   <si>
     <t>Venda - Parceria</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 690701025-102</t>
   </si>
 </sst>
 </file>
@@ -494,9 +497,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -534,7 +537,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -640,7 +643,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -782,7 +785,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -840,6 +843,21 @@
       <c r="A6" s="11" t="s">
         <v>26</v>
       </c>
+      <c r="B6" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="14">
+        <v>1650</v>
+      </c>
+      <c r="D6" s="13">
+        <v>46303</v>
+      </c>
+      <c r="E6" s="11">
+        <v>50</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
@@ -947,6 +965,12 @@
       </c>
       <c r="B15" s="11" t="s">
         <v>68</v>
+      </c>
+      <c r="C15" s="12">
+        <v>1350000</v>
+      </c>
+      <c r="D15" s="13">
+        <v>46303</v>
       </c>
       <c r="E15" s="11">
         <v>75</v>

</xml_diff>

<commit_message>
Atualiza painel (09/10/2026 18:02)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B97875DA-4664-46F2-8FBB-A3A4A3AB644A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00B2AEF2-A052-45BD-BA1A-5249A9FCF83B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="70">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -236,22 +236,6 @@
     <t>LOCAÇÃO - Cancelamento da captação de locação</t>
   </si>
   <si>
-    <t>690531104-966
-690531057-138</t>
-  </si>
-  <si>
-    <t>Locação  - Parceria
-Venda</t>
-  </si>
-  <si>
-    <t>R$ 4.400,00
-350.000,00</t>
-  </si>
-  <si>
-    <t>07/10/2026
-08/10/2026</t>
-  </si>
-  <si>
     <t>Locação</t>
   </si>
   <si>
@@ -265,6 +249,18 @@
   </si>
   <si>
     <t xml:space="preserve"> 690701025-102</t>
+  </si>
+  <si>
+    <t>Venda</t>
+  </si>
+  <si>
+    <t>Locação  - Parceria</t>
+  </si>
+  <si>
+    <t>690531057-138</t>
+  </si>
+  <si>
+    <t>690701039-6</t>
   </si>
 </sst>
 </file>
@@ -272,10 +268,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="8" formatCode="&quot;R$&quot;\ #,##0.00;[Red]\-&quot;R$&quot;\ #,##0.00"/>
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="dd/mm/\y\y\y\y"/>
     <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #.##000"/>
+    <numFmt numFmtId="166" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -387,7 +383,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -402,22 +398,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -427,12 +420,7 @@
   </cellStyles>
   <dxfs count="9">
     <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #.##000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #.##000"/>
-    </dxf>
-    <dxf>
+      <numFmt numFmtId="166" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -441,6 +429,12 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #.##000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #.##000"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -468,14 +462,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E53" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:E53" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E54" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:E54" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F68D7E3E-8D02-41D7-8907-35C934E19501}" name="Corretor" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{EACFDE5D-3403-4D4D-BD98-558F34E9A0F1}" name="Venda ou Locação" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{70453950-7621-41E3-A278-730F51464AA2}" name="Valor do Imóvel" dataDxfId="4" dataCellStyle="Moeda"/>
-    <tableColumn id="4" xr3:uid="{0B9D7A2A-7135-4189-AB83-E55B035B11A8}" name="Data da Captação" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{1AFC20BA-6A6F-459D-BBB9-5C9F2323A6AD}" name="Pontuação" dataDxfId="2">
+    <tableColumn id="2" xr3:uid="{EACFDE5D-3403-4D4D-BD98-558F34E9A0F1}" name="Venda ou Locação" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{70453950-7621-41E3-A278-730F51464AA2}" name="Valor do Imóvel" dataDxfId="0" dataCellStyle="Moeda"/>
+    <tableColumn id="4" xr3:uid="{0B9D7A2A-7135-4189-AB83-E55B035B11A8}" name="Data da Captação" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{1AFC20BA-6A6F-459D-BBB9-5C9F2323A6AD}" name="Pontuação" dataDxfId="5">
       <calculatedColumnFormula>IF(tbCaptacoes[[#This Row],[Valor do Imóvel]]="","",IFERROR(VLOOKUP(tbCaptacoes[[#This Row],[Valor do Imóvel]],tbFaixas[],3,TRUE),0))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -487,8 +481,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BE296B9A-7FB2-47EF-91CE-D94B7341102A}" name="tbFaixas" displayName="tbFaixas" ref="A1:D11" totalsRowShown="0">
   <autoFilter ref="A1:D11" xr:uid="{BE296B9A-7FB2-47EF-91CE-D94B7341102A}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{D2501A27-5A99-4009-8294-2BFD28385B1D}" name="Valor mínimo" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{488F6EEF-997C-45E1-B6E8-ADC37F785D66}" name="Valor máximo" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{D2501A27-5A99-4009-8294-2BFD28385B1D}" name="Valor mínimo" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{488F6EEF-997C-45E1-B6E8-ADC37F785D66}" name="Valor máximo" dataDxfId="3"/>
     <tableColumn id="3" xr3:uid="{830BDE7B-EA8B-4E6F-A7D4-9A97F158AED2}" name="Pontos"/>
     <tableColumn id="4" xr3:uid="{8056E5D0-FC15-43C2-A6CB-667290BADF20}" name="Faixa"/>
   </tableColumns>
@@ -497,9 +491,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -537,7 +531,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -643,7 +637,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -785,7 +779,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -797,8 +791,8 @@
   <sheetFormatPr defaultColWidth="26.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="26.44140625" style="11"/>
-    <col min="3" max="3" width="26.44140625" style="12"/>
-    <col min="4" max="4" width="26.44140625" style="13"/>
+    <col min="3" max="3" width="26.44140625" style="15"/>
+    <col min="4" max="4" width="26.44140625" style="12"/>
     <col min="5" max="16384" width="26.44140625" style="11"/>
   </cols>
   <sheetData>
@@ -809,10 +803,10 @@
       <c r="B1" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="12" t="s">
         <v>47</v>
       </c>
       <c r="E1" s="11" t="s">
@@ -844,19 +838,19 @@
         <v>26</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="C6" s="14">
+        <v>61</v>
+      </c>
+      <c r="C6" s="15">
         <v>1650</v>
       </c>
-      <c r="D6" s="13">
+      <c r="D6" s="12">
         <v>46303</v>
       </c>
       <c r="E6" s="11">
         <v>50</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -864,188 +858,220 @@
         <v>27</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="C7" s="14">
+        <v>64</v>
+      </c>
+      <c r="C7" s="15">
         <v>1350000</v>
       </c>
-      <c r="D7" s="13">
+      <c r="D7" s="12">
         <v>46303</v>
       </c>
       <c r="E7" s="11">
         <v>75</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="D8" s="17" t="s">
-        <v>64</v>
-      </c>
-      <c r="E8" s="15">
-        <v>135</v>
-      </c>
-      <c r="F8" s="15" t="s">
-        <v>61</v>
+      <c r="B8" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="C8" s="16">
+        <v>4400</v>
+      </c>
+      <c r="D8" s="14">
+        <v>46302</v>
+      </c>
+      <c r="E8" s="13">
+        <v>35</v>
+      </c>
+      <c r="F8" s="13" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
-        <v>38</v>
+        <v>20</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" s="16">
+        <v>350000</v>
+      </c>
+      <c r="D9" s="14">
+        <v>46303</v>
+      </c>
+      <c r="E9" s="13">
+        <v>100</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="C10" s="14">
-        <v>2190</v>
-      </c>
-      <c r="D10" s="13">
-        <v>46302</v>
-      </c>
-      <c r="E10" s="11">
-        <v>70</v>
-      </c>
-      <c r="F10" s="11" t="s">
-        <v>66</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" s="15">
+        <v>2190</v>
+      </c>
+      <c r="D11" s="12">
+        <v>46302</v>
+      </c>
+      <c r="E11" s="11">
+        <v>70</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="C12" s="14">
-        <v>4400</v>
-      </c>
-      <c r="D12" s="13">
-        <v>46302</v>
-      </c>
-      <c r="E12" s="11">
-        <v>35</v>
-      </c>
-      <c r="F12" s="11" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="15">
+        <v>4400</v>
+      </c>
+      <c r="D13" s="12">
+        <v>46302</v>
+      </c>
+      <c r="E13" s="11">
+        <v>35</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="C15" s="12">
-        <v>1350000</v>
-      </c>
-      <c r="D15" s="13">
-        <v>46303</v>
-      </c>
-      <c r="E15" s="11">
-        <v>75</v>
-      </c>
-      <c r="F15" s="11" t="s">
-        <v>67</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C16" s="15">
+        <v>1350000</v>
+      </c>
+      <c r="D16" s="12">
+        <v>46303</v>
+      </c>
+      <c r="E16" s="11">
+        <v>75</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="11" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="11" t="s">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="11" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="11" t="s">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="11" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="11" t="s">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="11" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="11" t="s">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="11" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="11" t="s">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="11" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="11" t="s">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="11" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="11" t="s">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="11" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="11" t="s">
+      <c r="B24" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C24" s="15">
+        <v>286200</v>
+      </c>
+      <c r="D24" s="12">
+        <v>46304</v>
+      </c>
+      <c r="E24" s="11">
+        <v>100</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="11" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="11" t="s">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="11" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="11" t="s">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="11" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="11" t="s">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="11" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="11" t="s">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" s="11" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C29" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>

<commit_message>
Atualiza painel (09/10/2026 18:08)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00B2AEF2-A052-45BD-BA1A-5249A9FCF83B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4011BEFA-A86F-4081-BEDB-B0C441DEAC3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="71">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -261,6 +261,9 @@
   </si>
   <si>
     <t>690701039-6</t>
+  </si>
+  <si>
+    <t>690531104-969</t>
   </si>
 </sst>
 </file>
@@ -462,8 +465,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E54" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:E54" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E55" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:E55" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F68D7E3E-8D02-41D7-8907-35C934E19501}" name="Corretor" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{EACFDE5D-3403-4D4D-BD98-558F34E9A0F1}" name="Venda ou Locação" dataDxfId="2"/>
@@ -787,7 +790,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51DF420C-6417-4C8E-9CA8-EAE7781FF48D}">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr defaultColWidth="26.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="26.44140625" style="11"/>
@@ -965,111 +968,131 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C14" s="15">
+        <v>2000</v>
+      </c>
+      <c r="D14" s="12">
+        <v>46304</v>
+      </c>
+      <c r="E14" s="11">
+        <v>50</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="C16" s="15">
-        <v>1350000</v>
-      </c>
-      <c r="D16" s="12">
-        <v>46303</v>
-      </c>
-      <c r="E16" s="11">
-        <v>75</v>
-      </c>
-      <c r="F16" s="11" t="s">
-        <v>63</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
-        <v>22</v>
+        <v>32</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C17" s="15">
+        <v>1350000</v>
+      </c>
+      <c r="D17" s="12">
+        <v>46303</v>
+      </c>
+      <c r="E17" s="11">
+        <v>75</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B24" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="C24" s="15">
-        <v>286200</v>
-      </c>
-      <c r="D24" s="12">
-        <v>46304</v>
-      </c>
-      <c r="E24" s="11">
-        <v>100</v>
-      </c>
-      <c r="F24" s="11" t="s">
-        <v>69</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C25" s="15">
+        <v>286200</v>
+      </c>
+      <c r="D25" s="12">
+        <v>46304</v>
+      </c>
+      <c r="E25" s="11">
+        <v>100</v>
+      </c>
+      <c r="F25" s="11" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" s="11" t="s">
         <v>46</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza painel (14/10/2026 14:49)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4011BEFA-A86F-4081-BEDB-B0C441DEAC3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C30AEF0E-2D45-4262-BFFD-58CA98894F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="82">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -264,6 +264,50 @@
   </si>
   <si>
     <t>690531104-969</t>
+  </si>
+  <si>
+    <t>Locação
+Locação - Parceria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.500,00
+R$ 72.000,00 </t>
+  </si>
+  <si>
+    <t>13/10/2026
+13/10/2026</t>
+  </si>
+  <si>
+    <t>70
+35</t>
+  </si>
+  <si>
+    <t>690531082-86
+690531082-89</t>
+  </si>
+  <si>
+    <t>690531082-89</t>
+  </si>
+  <si>
+    <t>Venda - Parceria
+Venda</t>
+  </si>
+  <si>
+    <t>1350000
+R$ 100.000,00</t>
+  </si>
+  <si>
+    <t>08/10/2026
+13/10/2026</t>
+  </si>
+  <si>
+    <t>75
+100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">690531008-310
+690531008-311
+</t>
   </si>
 </sst>
 </file>
@@ -423,7 +467,12 @@
   </cellStyles>
   <dxfs count="9">
     <dxf>
-      <numFmt numFmtId="166" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
+      <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #.##000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #.##000"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -431,13 +480,8 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="166" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #.##000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #.##000"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -469,10 +513,10 @@
   <autoFilter ref="A1:E55" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F68D7E3E-8D02-41D7-8907-35C934E19501}" name="Corretor" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{EACFDE5D-3403-4D4D-BD98-558F34E9A0F1}" name="Venda ou Locação" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{70453950-7621-41E3-A278-730F51464AA2}" name="Valor do Imóvel" dataDxfId="0" dataCellStyle="Moeda"/>
-    <tableColumn id="4" xr3:uid="{0B9D7A2A-7135-4189-AB83-E55B035B11A8}" name="Data da Captação" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{1AFC20BA-6A6F-459D-BBB9-5C9F2323A6AD}" name="Pontuação" dataDxfId="5">
+    <tableColumn id="2" xr3:uid="{EACFDE5D-3403-4D4D-BD98-558F34E9A0F1}" name="Venda ou Locação" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{70453950-7621-41E3-A278-730F51464AA2}" name="Valor do Imóvel" dataDxfId="4" dataCellStyle="Moeda"/>
+    <tableColumn id="4" xr3:uid="{0B9D7A2A-7135-4189-AB83-E55B035B11A8}" name="Data da Captação" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{1AFC20BA-6A6F-459D-BBB9-5C9F2323A6AD}" name="Pontuação" dataDxfId="2">
       <calculatedColumnFormula>IF(tbCaptacoes[[#This Row],[Valor do Imóvel]]="","",IFERROR(VLOOKUP(tbCaptacoes[[#This Row],[Valor do Imóvel]],tbFaixas[],3,TRUE),0))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -484,8 +528,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BE296B9A-7FB2-47EF-91CE-D94B7341102A}" name="tbFaixas" displayName="tbFaixas" ref="A1:D11" totalsRowShown="0">
   <autoFilter ref="A1:D11" xr:uid="{BE296B9A-7FB2-47EF-91CE-D94B7341102A}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{D2501A27-5A99-4009-8294-2BFD28385B1D}" name="Valor mínimo" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{488F6EEF-997C-45E1-B6E8-ADC37F785D66}" name="Valor máximo" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{D2501A27-5A99-4009-8294-2BFD28385B1D}" name="Valor mínimo" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{488F6EEF-997C-45E1-B6E8-ADC37F785D66}" name="Valor máximo" dataDxfId="0"/>
     <tableColumn id="3" xr3:uid="{830BDE7B-EA8B-4E6F-A7D4-9A97F158AED2}" name="Pontos"/>
     <tableColumn id="4" xr3:uid="{8056E5D0-FC15-43C2-A6CB-667290BADF20}" name="Faixa"/>
   </tableColumns>
@@ -494,9 +538,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -534,7 +578,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -640,7 +684,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -782,7 +826,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -835,6 +879,21 @@
       <c r="A5" s="11" t="s">
         <v>39</v>
       </c>
+      <c r="B5" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="15">
+        <v>72000</v>
+      </c>
+      <c r="D5" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E5" s="11">
+        <v>35</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
@@ -856,24 +915,24 @@
         <v>65</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="C7" s="15">
-        <v>1350000</v>
-      </c>
-      <c r="D7" s="12">
-        <v>46303</v>
-      </c>
-      <c r="E7" s="11">
-        <v>75</v>
-      </c>
-      <c r="F7" s="11" t="s">
-        <v>63</v>
+      <c r="B7" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -1036,9 +1095,24 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
         <v>36</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualiza painel (14/10/2026 14:59)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C30AEF0E-2D45-4262-BFFD-58CA98894F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E794AAC7-F754-43F9-A123-EE773B94C808}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="83">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -308,6 +308,9 @@
     <t xml:space="preserve">690531008-310
 690531008-311
 </t>
+  </si>
+  <si>
+    <t>690701024-233</t>
   </si>
 </sst>
 </file>
@@ -979,6 +982,18 @@
       <c r="A10" s="11" t="s">
         <v>38</v>
       </c>
+      <c r="B10" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" s="15">
+        <v>320000</v>
+      </c>
+      <c r="D10" s="12">
+        <v>46309</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">

</xml_diff>

<commit_message>
Atualiza painel (14/10/2026 15:05)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E794AAC7-F754-43F9-A123-EE773B94C808}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{367FDA19-2200-43EB-819B-62EF8353EC76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -991,6 +991,9 @@
       <c r="D10" s="12">
         <v>46309</v>
       </c>
+      <c r="E10" s="11">
+        <v>100</v>
+      </c>
       <c r="F10" s="11" t="s">
         <v>82</v>
       </c>

</xml_diff>

<commit_message>
Atualiza painel (14/10/2026 15:18)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{367FDA19-2200-43EB-819B-62EF8353EC76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4344F8D-074E-4985-A8B2-002DBA119A1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="84">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -311,6 +311,9 @@
   </si>
   <si>
     <t>690701024-233</t>
+  </si>
+  <si>
+    <t>690531094-36</t>
   </si>
 </sst>
 </file>
@@ -867,6 +870,21 @@
       <c r="A2" s="11" t="s">
         <v>23</v>
       </c>
+      <c r="B2" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" s="15">
+        <v>2000</v>
+      </c>
+      <c r="D2" s="12">
+        <v>46305</v>
+      </c>
+      <c r="E2" s="11">
+        <v>50</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
@@ -1071,6 +1089,9 @@
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
         <v>21</v>
+      </c>
+      <c r="E16" s="11">
+        <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualiza painel (14/10/2026 15:24)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4344F8D-074E-4985-A8B2-002DBA119A1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC0973F6-70CE-407D-AA87-7D2A27895403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -293,10 +293,6 @@
 Venda</t>
   </si>
   <si>
-    <t>1350000
-R$ 100.000,00</t>
-  </si>
-  <si>
     <t>08/10/2026
 13/10/2026</t>
   </si>
@@ -314,6 +310,10 @@
   </si>
   <si>
     <t>690531094-36</t>
+  </si>
+  <si>
+    <t>R$ 1.350.000,00
+R$ 100.000,00</t>
   </si>
 </sst>
 </file>
@@ -883,7 +883,7 @@
         <v>50</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -944,16 +944,16 @@
         <v>77</v>
       </c>
       <c r="C7" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="D7" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="E7" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="F7" s="13" t="s">
         <v>80</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -1013,7 +1013,7 @@
         <v>100</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualiza painel (14/10/2026 15:30)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC0973F6-70CE-407D-AA87-7D2A27895403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F0596AE-F89A-44EB-97E6-3521835AEA56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="82">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -278,10 +278,6 @@
 13/10/2026</t>
   </si>
   <si>
-    <t>70
-35</t>
-  </si>
-  <si>
     <t>690531082-86
 690531082-89</t>
   </si>
@@ -295,10 +291,6 @@
   <si>
     <t>08/10/2026
 13/10/2026</t>
-  </si>
-  <si>
-    <t>75
-100</t>
   </si>
   <si>
     <t xml:space="preserve">690531008-310
@@ -883,7 +875,7 @@
         <v>50</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -913,7 +905,7 @@
         <v>35</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -941,19 +933,19 @@
         <v>27</v>
       </c>
       <c r="B7" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="D7" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="C7" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="D7" s="14" t="s">
+      <c r="E7" s="13">
+        <v>175</v>
+      </c>
+      <c r="F7" s="13" t="s">
         <v>78</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -1013,7 +1005,7 @@
         <v>100</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -1147,11 +1139,11 @@
       <c r="D22" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="E22" s="13" t="s">
+      <c r="E22" s="13">
+        <v>105</v>
+      </c>
+      <c r="F22" s="13" t="s">
         <v>74</v>
-      </c>
-      <c r="F22" s="13" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualiza painel (14/10/2026 15:44)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46155CE0-FBBB-4D5A-BD9A-BB74CC74B27D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BB7428B-C9AC-4C34-A841-73827FD65756}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="85">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -143,9 +143,6 @@
     <t>Oseias Amorim</t>
   </si>
   <si>
-    <t>Rafael Gil</t>
-  </si>
-  <si>
     <t>Rayane Fontoura</t>
   </si>
   <si>
@@ -261,9 +258,6 @@
   </si>
   <si>
     <t>690701039-6</t>
-  </si>
-  <si>
-    <t>690531104-969</t>
   </si>
   <si>
     <t>Locação
@@ -306,6 +300,26 @@
   <si>
     <t>R$ 1.350.000,00
 R$ 100.000,00</t>
+  </si>
+  <si>
+    <t>Rafael Gil
+Rafael Gil</t>
+  </si>
+  <si>
+    <t>Locação - Parceria
+Locação</t>
+  </si>
+  <si>
+    <t>4.400,00
+R$ 2.000,00</t>
+  </si>
+  <si>
+    <t>07/10/2026
+09/10/2026</t>
+  </si>
+  <si>
+    <t>690531104-966
+690531104-969</t>
   </si>
 </sst>
 </file>
@@ -507,8 +521,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E55" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:E55" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E54" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:E54" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F68D7E3E-8D02-41D7-8907-35C934E19501}" name="Corretor" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{EACFDE5D-3403-4D4D-BD98-558F34E9A0F1}" name="Venda ou Locação" dataDxfId="5"/>
@@ -832,7 +846,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51DF420C-6417-4C8E-9CA8-EAE7781FF48D}">
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr defaultColWidth="26.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="26.44140625" style="11"/>
@@ -846,13 +860,13 @@
         <v>15</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C1" s="15" t="s">
         <v>16</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E1" s="11" t="s">
         <v>17</v>
@@ -863,7 +877,7 @@
         <v>23</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C2" s="15">
         <v>2000</v>
@@ -875,7 +889,7 @@
         <v>50</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -890,10 +904,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C5" s="15">
         <v>72000</v>
@@ -905,7 +919,7 @@
         <v>35</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -913,7 +927,7 @@
         <v>26</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C6" s="15">
         <v>1650</v>
@@ -925,7 +939,7 @@
         <v>50</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
@@ -933,19 +947,19 @@
         <v>27</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E7" s="13">
         <v>175</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -953,7 +967,7 @@
         <v>20</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C8" s="16">
         <v>4400</v>
@@ -965,7 +979,7 @@
         <v>35</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -973,7 +987,7 @@
         <v>20</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C9" s="16">
         <v>350000</v>
@@ -985,15 +999,15 @@
         <v>100</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C10" s="15">
         <v>320000</v>
@@ -1005,7 +1019,7 @@
         <v>100</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -1013,7 +1027,7 @@
         <v>28</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C11" s="15">
         <v>2190</v>
@@ -1025,7 +1039,7 @@
         <v>70</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -1033,82 +1047,67 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="C13" s="15">
-        <v>4400</v>
-      </c>
-      <c r="D13" s="12">
-        <v>46302</v>
+    <row r="13" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>83</v>
       </c>
       <c r="E13" s="11">
-        <v>35</v>
-      </c>
-      <c r="F13" s="11" t="s">
-        <v>50</v>
+        <v>85</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="C14" s="15">
-        <v>2000</v>
-      </c>
-      <c r="D14" s="12">
-        <v>46304</v>
-      </c>
-      <c r="E14" s="11">
-        <v>50</v>
-      </c>
-      <c r="F14" s="11" t="s">
-        <v>70</v>
-      </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
-        <v>31</v>
+        <v>21</v>
+      </c>
+      <c r="E15" s="11">
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
-        <v>21</v>
+        <v>31</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C16" s="15">
+        <v>1350000</v>
+      </c>
+      <c r="D16" s="12">
+        <v>46303</v>
       </c>
       <c r="E16" s="11">
-        <v>100</v>
+        <v>75</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="C17" s="15">
-        <v>1350000</v>
-      </c>
-      <c r="D17" s="12">
-        <v>46303</v>
-      </c>
-      <c r="E17" s="11">
-        <v>75</v>
-      </c>
-      <c r="F17" s="11" t="s">
-        <v>63</v>
+        <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -1121,60 +1120,60 @@
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B21" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="E21" s="13">
+        <v>105</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B22" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="C22" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="D22" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="E22" s="13">
-        <v>105</v>
-      </c>
-      <c r="F22" s="13" t="s">
-        <v>74</v>
-      </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
         <v>40</v>
       </c>
+      <c r="B24" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C24" s="15">
+        <v>286200</v>
+      </c>
+      <c r="D24" s="12">
+        <v>46304</v>
+      </c>
+      <c r="E24" s="11">
+        <v>100</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B25" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="C25" s="15">
-        <v>286200</v>
-      </c>
-      <c r="D25" s="12">
-        <v>46304</v>
-      </c>
-      <c r="E25" s="11">
-        <v>100</v>
-      </c>
-      <c r="F25" s="11" t="s">
-        <v>69</v>
-      </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
@@ -1194,11 +1193,6 @@
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="s">
         <v>45</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="11" t="s">
-        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -1242,7 +1236,7 @@
         <v>100</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -1252,7 +1246,7 @@
         <v>130</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -1262,7 +1256,7 @@
         <v>120</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -1272,7 +1266,7 @@
         <v>150</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -1282,7 +1276,7 @@
         <v>50</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -1292,7 +1286,7 @@
         <v>-50</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -1302,7 +1296,7 @@
         <v>200</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -1312,7 +1306,7 @@
         <v>50</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -1322,7 +1316,7 @@
         <v>70</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -1332,7 +1326,7 @@
         <v>-50</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualiza painel (14/10/2026 16:19)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEEA6851-E37A-4CFE-A328-46EAF6B64FD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{255978E0-F927-4396-A030-0DF189C76BB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -21,6 +21,17 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -51,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="76">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -143,6 +154,9 @@
     <t>Oseias Amorim</t>
   </si>
   <si>
+    <t>Rafael Gil</t>
+  </si>
+  <si>
     <t>Rayane Fontoura</t>
   </si>
   <si>
@@ -260,66 +274,22 @@
     <t>690701039-6</t>
   </si>
   <si>
-    <t>Locação
-Locação - Parceria</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.500,00
-R$ 72.000,00 </t>
-  </si>
-  <si>
-    <t>13/10/2026
-13/10/2026</t>
-  </si>
-  <si>
-    <t>690531082-86
-690531082-89</t>
+    <t>690531104-969</t>
+  </si>
+  <si>
+    <t>690531082-86</t>
   </si>
   <si>
     <t>690531082-89</t>
   </si>
   <si>
-    <t>Venda - Parceria
-Venda</t>
-  </si>
-  <si>
-    <t>08/10/2026
-13/10/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">690531008-310
-690531008-311
-</t>
-  </si>
-  <si>
     <t>690701024-233</t>
   </si>
   <si>
     <t>690531094-36</t>
   </si>
   <si>
-    <t>R$ 1.350.000,00
-R$ 100.000,00</t>
-  </si>
-  <si>
-    <t>Rafael Gil
-Rafael Gil</t>
-  </si>
-  <si>
-    <t>Locação - Parceria
-Locação</t>
-  </si>
-  <si>
-    <t>4.400,00
-R$ 2.000,00</t>
-  </si>
-  <si>
-    <t>07/10/2026
-09/10/2026</t>
-  </si>
-  <si>
-    <t>690531104-966
-690531104-969</t>
+    <t>690531008-311</t>
   </si>
 </sst>
 </file>
@@ -521,8 +491,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E54" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:E54" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E57" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:E57" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F68D7E3E-8D02-41D7-8907-35C934E19501}" name="Corretor" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{EACFDE5D-3403-4D4D-BD98-558F34E9A0F1}" name="Venda ou Locação" dataDxfId="5"/>
@@ -846,7 +816,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51DF420C-6417-4C8E-9CA8-EAE7781FF48D}">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultColWidth="26.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="26.44140625" style="11"/>
@@ -860,13 +830,13 @@
         <v>15</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C1" s="15" t="s">
         <v>16</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E1" s="11" t="s">
         <v>17</v>
@@ -877,7 +847,7 @@
         <v>23</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C2" s="15">
         <v>2000</v>
@@ -889,7 +859,7 @@
         <v>50</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -904,10 +874,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C5" s="15">
         <v>72000</v>
@@ -919,7 +889,7 @@
         <v>35</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -927,7 +897,7 @@
         <v>26</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C6" s="15">
         <v>1650</v>
@@ -939,260 +909,320 @@
         <v>50</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
         <v>27</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="D7" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="C7" s="16">
+        <v>1350000</v>
+      </c>
+      <c r="D7" s="14">
+        <v>46303</v>
+      </c>
+      <c r="E7" s="13">
         <v>75</v>
       </c>
-      <c r="E7" s="13">
-        <v>175</v>
-      </c>
       <c r="F7" s="13" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="C8" s="16">
-        <v>4400</v>
-      </c>
-      <c r="D8" s="14">
-        <v>46302</v>
-      </c>
-      <c r="E8" s="13">
-        <v>35</v>
+      <c r="C8" s="15">
+        <v>100000</v>
+      </c>
+      <c r="D8" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E8" s="11">
+        <v>100</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C9" s="16">
-        <v>350000</v>
+        <v>4400</v>
       </c>
       <c r="D9" s="14">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E9" s="13">
-        <v>100</v>
+        <v>35</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>67</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="C10" s="15">
-        <v>320000</v>
-      </c>
-      <c r="D10" s="12">
-        <v>46309</v>
-      </c>
-      <c r="E10" s="11">
+        <v>20</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" s="16">
+        <v>350000</v>
+      </c>
+      <c r="D10" s="14">
+        <v>46303</v>
+      </c>
+      <c r="E10" s="13">
         <v>100</v>
       </c>
-      <c r="F10" s="11" t="s">
-        <v>77</v>
+      <c r="F10" s="13" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="C11" s="15">
-        <v>2190</v>
+        <v>320000</v>
       </c>
       <c r="D11" s="12">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="E11" s="11">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" s="15">
+        <v>2190</v>
+      </c>
+      <c r="D12" s="12">
+        <v>46302</v>
+      </c>
+      <c r="E12" s="11">
+        <v>70</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="11" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="B13" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="C13" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="D13" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="E13" s="11">
-        <v>85</v>
-      </c>
-      <c r="F13" s="13" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
         <v>30</v>
       </c>
+      <c r="B14" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="C14" s="15">
+        <v>4400</v>
+      </c>
+      <c r="D14" s="12">
+        <v>46302</v>
+      </c>
+      <c r="E14" s="11">
+        <v>35</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
-        <v>21</v>
+        <v>30</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C15" s="15">
+        <v>2000</v>
+      </c>
+      <c r="D15" s="12">
+        <v>46304</v>
       </c>
       <c r="E15" s="11">
-        <v>100</v>
+        <v>50</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="C16" s="15">
-        <v>1350000</v>
-      </c>
-      <c r="D16" s="12">
-        <v>46303</v>
-      </c>
-      <c r="E16" s="11">
-        <v>75</v>
-      </c>
-      <c r="F16" s="11" t="s">
-        <v>62</v>
-      </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
+      </c>
+      <c r="E17" s="11">
+        <v>100</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
         <v>32</v>
       </c>
+      <c r="B18" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C18" s="15">
+        <v>1350000</v>
+      </c>
+      <c r="D18" s="12">
+        <v>46303</v>
+      </c>
+      <c r="E18" s="11">
+        <v>75</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="11" t="s">
         <v>34</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A21" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="B21" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="C21" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="D21" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="E21" s="13">
-        <v>105</v>
-      </c>
-      <c r="F21" s="13" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
-        <v>39</v>
+        <v>36</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C23" s="16">
+        <v>6500</v>
+      </c>
+      <c r="D23" s="14">
+        <v>46308</v>
+      </c>
+      <c r="E23" s="13">
+        <v>75</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="C24" s="15">
-        <v>286200</v>
+        <v>72000</v>
       </c>
       <c r="D24" s="12">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="E24" s="11">
-        <v>100</v>
-      </c>
-      <c r="F24" s="11" t="s">
-        <v>68</v>
+        <v>35</v>
+      </c>
+      <c r="F24" s="13" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="11" t="s">
-        <v>43</v>
+        <v>41</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C27" s="15">
+        <v>286200</v>
+      </c>
+      <c r="D27" s="12">
+        <v>46304</v>
+      </c>
+      <c r="E27" s="11">
+        <v>100</v>
+      </c>
+      <c r="F27" s="11" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" s="11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" s="11" t="s">
         <v>45</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="11" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -1236,7 +1266,7 @@
         <v>100</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -1246,7 +1276,7 @@
         <v>130</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -1256,7 +1286,7 @@
         <v>120</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -1266,7 +1296,7 @@
         <v>150</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -1276,7 +1306,7 @@
         <v>50</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -1286,7 +1316,7 @@
         <v>-50</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -1296,7 +1326,7 @@
         <v>200</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -1306,7 +1336,7 @@
         <v>50</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -1316,7 +1346,7 @@
         <v>70</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -1326,7 +1356,7 @@
         <v>-50</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualiza painel (14/10/2026 17:53)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{255978E0-F927-4396-A030-0DF189C76BB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36391A1B-3A3F-495F-84BD-0F1760846580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="78">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -290,6 +290,12 @@
   </si>
   <si>
     <t>690531008-311</t>
+  </si>
+  <si>
+    <t>690701039-8</t>
+  </si>
+  <si>
+    <t>690701039-7</t>
   </si>
 </sst>
 </file>
@@ -491,8 +497,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E57" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:E57" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E59" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:E59" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F68D7E3E-8D02-41D7-8907-35C934E19501}" name="Corretor" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{EACFDE5D-3403-4D4D-BD98-558F34E9A0F1}" name="Venda ou Locação" dataDxfId="5"/>
@@ -816,7 +822,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51DF420C-6417-4C8E-9CA8-EAE7781FF48D}">
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr defaultColWidth="26.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="26.44140625" style="11"/>
@@ -1202,26 +1208,66 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C28" s="15">
+        <v>16000</v>
+      </c>
+      <c r="D28" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E28" s="11">
+        <v>70</v>
+      </c>
+      <c r="F28" s="11" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="s">
-        <v>43</v>
+        <v>41</v>
+      </c>
+      <c r="B29" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" s="15">
+        <v>8000</v>
+      </c>
+      <c r="D29" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E29" s="11">
+        <v>70</v>
+      </c>
+      <c r="F29" s="11" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="11" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A33" s="11" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A34" s="11" t="s">
         <v>46</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza painel (14/10/2026 18:05)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CAD0FB5-F95A-4C52-B3EF-704CBFD54B13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBB509EC-9E1F-4BC7-9277-0E497ADCBE4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -1092,9 +1092,6 @@
       <c r="A17" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="E17" s="11">
-        <v>100</v>
-      </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">

</xml_diff>

<commit_message>
Atualiza painel (15/10/2026 13:43)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBB509EC-9E1F-4BC7-9277-0E497ADCBE4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{909491EB-B4B4-4B4D-84CB-19D402BC0287}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="82">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -296,6 +296,18 @@
   </si>
   <si>
     <t>690701039-7</t>
+  </si>
+  <si>
+    <t>690701039-10</t>
+  </si>
+  <si>
+    <t>690701039-9</t>
+  </si>
+  <si>
+    <t>690701039-12</t>
+  </si>
+  <si>
+    <t>690531082-90</t>
   </si>
 </sst>
 </file>
@@ -497,8 +509,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E59" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:E59" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E64" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:E64" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F68D7E3E-8D02-41D7-8907-35C934E19501}" name="Corretor" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{EACFDE5D-3403-4D4D-BD98-558F34E9A0F1}" name="Venda ou Locação" dataDxfId="5"/>
@@ -822,7 +834,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51DF420C-6417-4C8E-9CA8-EAE7781FF48D}">
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr defaultColWidth="26.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="26.44140625" style="11"/>
@@ -886,7 +898,7 @@
         <v>49</v>
       </c>
       <c r="C5" s="15">
-        <v>72000</v>
+        <v>73000</v>
       </c>
       <c r="D5" s="12">
         <v>46308</v>
@@ -958,109 +970,109 @@
         <v>75</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="C9" s="16">
-        <v>4400</v>
-      </c>
-      <c r="D9" s="14">
-        <v>46302</v>
-      </c>
-      <c r="E9" s="13">
-        <v>35</v>
+        <v>27</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C9" s="15">
+        <v>450000</v>
+      </c>
+      <c r="D9" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E9" s="11">
+        <v>50</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
         <v>20</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C10" s="16">
-        <v>350000</v>
+        <v>4400</v>
       </c>
       <c r="D10" s="14">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E10" s="13">
-        <v>100</v>
+        <v>35</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="C11" s="15">
-        <v>320000</v>
-      </c>
-      <c r="D11" s="12">
-        <v>46309</v>
-      </c>
-      <c r="E11" s="11">
+      <c r="C11" s="16">
+        <v>350000</v>
+      </c>
+      <c r="D11" s="14">
+        <v>46303</v>
+      </c>
+      <c r="E11" s="13">
         <v>100</v>
       </c>
-      <c r="F11" s="11" t="s">
-        <v>73</v>
+      <c r="F11" s="13" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C12" s="15">
-        <v>2190</v>
+        <v>320000</v>
       </c>
       <c r="D12" s="12">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="E12" s="11">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>62</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" s="15">
+        <v>2190</v>
+      </c>
+      <c r="D13" s="12">
+        <v>46302</v>
+      </c>
+      <c r="E13" s="11">
+        <v>70</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="C14" s="15">
-        <v>4400</v>
-      </c>
-      <c r="D14" s="12">
-        <v>46302</v>
-      </c>
-      <c r="E14" s="11">
-        <v>35</v>
-      </c>
-      <c r="F14" s="11" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -1068,159 +1080,159 @@
         <v>30</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="C15" s="15">
-        <v>2000</v>
+        <v>4400</v>
       </c>
       <c r="D15" s="12">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="E15" s="11">
+        <v>35</v>
+      </c>
+      <c r="F15" s="11" t="s">
         <v>50</v>
-      </c>
-      <c r="F15" s="11" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" s="15">
+        <v>2000</v>
+      </c>
+      <c r="D16" s="12">
+        <v>46304</v>
+      </c>
+      <c r="E16" s="11">
+        <v>50</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="C18" s="15">
-        <v>1350000</v>
-      </c>
-      <c r="D18" s="12">
-        <v>46303</v>
-      </c>
-      <c r="E18" s="11">
-        <v>75</v>
-      </c>
-      <c r="F18" s="11" t="s">
-        <v>63</v>
+        <v>21</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
-        <v>22</v>
+        <v>32</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C19" s="15">
+        <v>1350000</v>
+      </c>
+      <c r="D19" s="12">
+        <v>46303</v>
+      </c>
+      <c r="E19" s="11">
+        <v>75</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B23" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="C23" s="16">
-        <v>6500</v>
-      </c>
-      <c r="D23" s="14">
-        <v>46308</v>
-      </c>
-      <c r="E23" s="13">
-        <v>75</v>
-      </c>
-      <c r="F23" s="13" t="s">
-        <v>71</v>
+        <v>35</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B24" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="C24" s="15">
-        <v>72000</v>
-      </c>
-      <c r="D24" s="12">
+      <c r="B24" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C24" s="16">
+        <v>6500</v>
+      </c>
+      <c r="D24" s="14">
         <v>46308</v>
       </c>
-      <c r="E24" s="11">
-        <v>35</v>
+      <c r="E24" s="13">
+        <v>75</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" s="15">
+        <v>73000</v>
+      </c>
+      <c r="D25" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E25" s="11">
+        <v>35</v>
+      </c>
+      <c r="F25" s="13" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
-        <v>40</v>
+        <v>36</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C26" s="15">
+        <v>450000</v>
+      </c>
+      <c r="D26" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E26" s="11">
+        <v>50</v>
+      </c>
+      <c r="F26" s="13" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B27" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="C27" s="15">
-        <v>286200</v>
-      </c>
-      <c r="D27" s="12">
-        <v>46304</v>
-      </c>
-      <c r="E27" s="11">
-        <v>100</v>
-      </c>
-      <c r="F27" s="11" t="s">
-        <v>69</v>
+        <v>37</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B28" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="C28" s="15">
-        <v>16000</v>
-      </c>
-      <c r="D28" s="12">
-        <v>46309</v>
-      </c>
-      <c r="E28" s="11">
-        <v>70</v>
-      </c>
-      <c r="F28" s="11" t="s">
-        <v>76</v>
+        <v>40</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
@@ -1228,52 +1240,153 @@
         <v>41</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C29" s="15">
-        <v>8000</v>
+        <v>286200</v>
       </c>
       <c r="D29" s="12">
-        <v>46309</v>
+        <v>46304</v>
       </c>
       <c r="E29" s="11">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
+      </c>
+      <c r="B30" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C30" s="15">
+        <v>16000</v>
+      </c>
+      <c r="D30" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E30" s="11">
+        <v>70</v>
+      </c>
+      <c r="F30" s="11" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="11" t="s">
-        <v>43</v>
+        <v>41</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C31" s="15">
+        <v>8000</v>
+      </c>
+      <c r="D31" s="12">
+        <v>46310</v>
+      </c>
+      <c r="E31" s="11">
+        <v>70</v>
+      </c>
+      <c r="F31" s="11" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B32" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C32" s="15">
+        <v>80000</v>
+      </c>
+      <c r="D32" s="12">
+        <v>46310</v>
+      </c>
+      <c r="E32" s="11">
+        <v>100</v>
+      </c>
+      <c r="F32" s="11" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C33" s="15">
+        <v>1650</v>
+      </c>
+      <c r="D33" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E33" s="11">
+        <v>50</v>
+      </c>
+      <c r="F33" s="11" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B34" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C34" s="15">
+        <v>8000</v>
+      </c>
+      <c r="D34" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E34" s="11">
+        <v>70</v>
+      </c>
+      <c r="F34" s="11" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" s="11" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" s="11" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A33" s="11" t="s">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" s="11" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A34" s="11" t="s">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" s="11" t="s">
         <v>46</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Atualiza painel (19/10/2026 14:24)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{909491EB-B4B4-4B4D-84CB-19D402BC0287}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8591528F-50F3-4585-8E0A-75C33CB9C3FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="85">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -308,6 +308,15 @@
   </si>
   <si>
     <t>690531082-90</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 690531104-970</t>
+  </si>
+  <si>
+    <t>690531126-47</t>
+  </si>
+  <si>
+    <t>690701043-2</t>
   </si>
 </sst>
 </file>
@@ -509,8 +518,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E64" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:E64" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E65" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:E65" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F68D7E3E-8D02-41D7-8907-35C934E19501}" name="Corretor" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{EACFDE5D-3403-4D4D-BD98-558F34E9A0F1}" name="Venda ou Locação" dataDxfId="5"/>
@@ -834,7 +843,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51DF420C-6417-4C8E-9CA8-EAE7781FF48D}">
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr defaultColWidth="26.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="26.44140625" style="11"/>
@@ -889,6 +898,21 @@
       <c r="A4" s="11" t="s">
         <v>25</v>
       </c>
+      <c r="B4" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4" s="15">
+        <v>185000</v>
+      </c>
+      <c r="D4" s="12">
+        <v>46310</v>
+      </c>
+      <c r="E4" s="11">
+        <v>100</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
@@ -1117,92 +1141,92 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" s="15">
+        <v>2100</v>
+      </c>
+      <c r="D17" s="12">
+        <v>46310</v>
+      </c>
+      <c r="E17" s="11">
+        <v>70</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="C19" s="15">
-        <v>1350000</v>
-      </c>
-      <c r="D19" s="12">
-        <v>46303</v>
-      </c>
-      <c r="E19" s="11">
-        <v>75</v>
-      </c>
-      <c r="F19" s="11" t="s">
-        <v>63</v>
+        <v>21</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
-        <v>22</v>
+        <v>32</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C20" s="15">
+        <v>1350000</v>
+      </c>
+      <c r="D20" s="12">
+        <v>46303</v>
+      </c>
+      <c r="E20" s="11">
+        <v>75</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B24" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="C24" s="16">
-        <v>6500</v>
-      </c>
-      <c r="D24" s="14">
-        <v>46308</v>
-      </c>
-      <c r="E24" s="13">
-        <v>75</v>
-      </c>
-      <c r="F24" s="13" t="s">
-        <v>71</v>
+        <v>35</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B25" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="C25" s="15">
-        <v>73000</v>
-      </c>
-      <c r="D25" s="12">
+      <c r="B25" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C25" s="16">
+        <v>6500</v>
+      </c>
+      <c r="D25" s="14">
         <v>46308</v>
       </c>
-      <c r="E25" s="11">
-        <v>35</v>
+      <c r="E25" s="13">
+        <v>75</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
@@ -1210,49 +1234,49 @@
         <v>36</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="C26" s="15">
-        <v>450000</v>
+        <v>73000</v>
       </c>
       <c r="D26" s="12">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="E26" s="11">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="F26" s="13" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C27" s="15">
+        <v>450000</v>
+      </c>
+      <c r="D27" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E27" s="11">
+        <v>50</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B29" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="C29" s="15">
-        <v>286200</v>
-      </c>
-      <c r="D29" s="12">
-        <v>46304</v>
-      </c>
-      <c r="E29" s="11">
-        <v>100</v>
-      </c>
-      <c r="F29" s="11" t="s">
-        <v>69</v>
+        <v>40</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
@@ -1260,19 +1284,19 @@
         <v>41</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C30" s="15">
-        <v>16000</v>
+        <v>286200</v>
       </c>
       <c r="D30" s="12">
-        <v>46309</v>
+        <v>46304</v>
       </c>
       <c r="E30" s="11">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
@@ -1283,16 +1307,16 @@
         <v>61</v>
       </c>
       <c r="C31" s="15">
-        <v>8000</v>
+        <v>16000</v>
       </c>
       <c r="D31" s="12">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="E31" s="11">
         <v>70</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
@@ -1300,19 +1324,19 @@
         <v>41</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C32" s="15">
-        <v>80000</v>
+        <v>8000</v>
       </c>
       <c r="D32" s="12">
         <v>46310</v>
       </c>
       <c r="E32" s="11">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
@@ -1320,19 +1344,19 @@
         <v>41</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C33" s="15">
-        <v>1650</v>
+        <v>80000</v>
       </c>
       <c r="D33" s="12">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="E33" s="11">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
@@ -1343,40 +1367,75 @@
         <v>61</v>
       </c>
       <c r="C34" s="15">
-        <v>8000</v>
+        <v>1650</v>
       </c>
       <c r="D34" s="12">
         <v>46309</v>
       </c>
       <c r="E34" s="11">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
+      </c>
+      <c r="B35" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C35" s="15">
+        <v>8000</v>
+      </c>
+      <c r="D35" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E35" s="11">
+        <v>70</v>
+      </c>
+      <c r="F35" s="11" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B39" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C39" s="15">
+        <v>125000</v>
+      </c>
+      <c r="D39" s="12">
+        <v>46311</v>
+      </c>
+      <c r="E39" s="11">
+        <v>100</v>
+      </c>
+      <c r="F39" s="11" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" s="11" t="s">
         <v>46</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza painel (20/10/2026 10:43)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8591528F-50F3-4585-8E0A-75C33CB9C3FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68E522AD-9860-4F6A-BD2D-39DA48FFFC2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="90">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -317,6 +317,21 @@
   </si>
   <si>
     <t>690701043-2</t>
+  </si>
+  <si>
+    <t>690531104-971</t>
+  </si>
+  <si>
+    <t>690701036-77</t>
+  </si>
+  <si>
+    <t>690701021-158</t>
+  </si>
+  <si>
+    <t>690531008-313</t>
+  </si>
+  <si>
+    <t>690531126-48</t>
   </si>
 </sst>
 </file>
@@ -518,8 +533,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E65" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:E65" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E69" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:E69" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F68D7E3E-8D02-41D7-8907-35C934E19501}" name="Corretor" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{EACFDE5D-3403-4D4D-BD98-558F34E9A0F1}" name="Venda ou Locação" dataDxfId="5"/>
@@ -843,7 +858,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51DF420C-6417-4C8E-9CA8-EAE7781FF48D}">
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr defaultColWidth="26.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="26.44140625" style="11"/>
@@ -916,82 +931,82 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="C5" s="15">
-        <v>73000</v>
+        <v>1500</v>
       </c>
       <c r="D5" s="12">
-        <v>46308</v>
+        <v>46314</v>
       </c>
       <c r="E5" s="11">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="C6" s="15">
-        <v>1650</v>
+        <v>73000</v>
       </c>
       <c r="D6" s="12">
-        <v>46303</v>
+        <v>46308</v>
       </c>
       <c r="E6" s="11">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="C7" s="16">
-        <v>1350000</v>
-      </c>
-      <c r="D7" s="14">
+        <v>26</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" s="15">
+        <v>1650</v>
+      </c>
+      <c r="D7" s="12">
         <v>46303</v>
       </c>
-      <c r="E7" s="13">
-        <v>75</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>63</v>
+      <c r="E7" s="11">
+        <v>50</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="C8" s="15">
-        <v>100000</v>
-      </c>
-      <c r="D8" s="12">
-        <v>46308</v>
-      </c>
-      <c r="E8" s="11">
-        <v>100</v>
+      <c r="B8" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8" s="16">
+        <v>1350000</v>
+      </c>
+      <c r="D8" s="14">
+        <v>46303</v>
+      </c>
+      <c r="E8" s="13">
+        <v>75</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -999,364 +1014,376 @@
         <v>27</v>
       </c>
       <c r="B9" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" s="15">
+        <v>100000</v>
+      </c>
+      <c r="D9" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E9" s="11">
+        <v>100</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="C9" s="15">
+      <c r="C10" s="15">
         <v>450000</v>
       </c>
-      <c r="D9" s="12">
+      <c r="D10" s="12">
         <v>46309</v>
       </c>
-      <c r="E9" s="11">
+      <c r="E10" s="11">
         <v>50</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F10" s="13" t="s">
         <v>81</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="C10" s="16">
-        <v>4400</v>
-      </c>
-      <c r="D10" s="14">
-        <v>46302</v>
-      </c>
-      <c r="E10" s="13">
-        <v>35</v>
-      </c>
-      <c r="F10" s="13" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" s="15">
+        <v>1700</v>
+      </c>
+      <c r="D11" s="12">
+        <v>46315</v>
+      </c>
+      <c r="E11" s="11">
+        <v>50</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="C11" s="16">
-        <v>350000</v>
-      </c>
-      <c r="D11" s="14">
-        <v>46303</v>
-      </c>
-      <c r="E11" s="13">
-        <v>100</v>
-      </c>
-      <c r="F11" s="13" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="C12" s="15">
-        <v>320000</v>
-      </c>
-      <c r="D12" s="12">
-        <v>46309</v>
-      </c>
-      <c r="E12" s="11">
-        <v>100</v>
-      </c>
-      <c r="F12" s="11" t="s">
-        <v>73</v>
+      <c r="B12" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" s="16">
+        <v>4400</v>
+      </c>
+      <c r="D12" s="14">
+        <v>46302</v>
+      </c>
+      <c r="E12" s="13">
+        <v>35</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="C13" s="15">
-        <v>2190</v>
-      </c>
-      <c r="D13" s="12">
-        <v>46302</v>
-      </c>
-      <c r="E13" s="11">
-        <v>70</v>
-      </c>
-      <c r="F13" s="11" t="s">
-        <v>62</v>
+        <v>20</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="C13" s="16">
+        <v>350000</v>
+      </c>
+      <c r="D13" s="14">
+        <v>46303</v>
+      </c>
+      <c r="E13" s="13">
+        <v>100</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
-        <v>29</v>
+        <v>38</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="15">
+        <v>320000</v>
+      </c>
+      <c r="D14" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E14" s="11">
+        <v>100</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="C15" s="15">
-        <v>4400</v>
+        <v>2190</v>
       </c>
       <c r="D15" s="12">
         <v>46302</v>
       </c>
       <c r="E15" s="11">
-        <v>35</v>
+        <v>70</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C16" s="15">
-        <v>2000</v>
-      </c>
-      <c r="D16" s="12">
-        <v>46304</v>
+        <v>2100000</v>
       </c>
       <c r="E16" s="11">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="C17" s="15">
-        <v>2100</v>
-      </c>
-      <c r="D17" s="12">
-        <v>46310</v>
-      </c>
-      <c r="E17" s="11">
-        <v>70</v>
-      </c>
-      <c r="F17" s="11" t="s">
-        <v>82</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" s="15">
+        <v>4400</v>
+      </c>
+      <c r="D18" s="12">
+        <v>46302</v>
+      </c>
+      <c r="E18" s="11">
+        <v>35</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
-        <v>21</v>
+        <v>30</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C19" s="15">
+        <v>2000</v>
+      </c>
+      <c r="D19" s="12">
+        <v>46304</v>
+      </c>
+      <c r="E19" s="11">
+        <v>50</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C20" s="15">
-        <v>1350000</v>
+        <v>2100</v>
       </c>
       <c r="D20" s="12">
-        <v>46303</v>
+        <v>46310</v>
       </c>
       <c r="E20" s="11">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>63</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
-        <v>22</v>
+        <v>30</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" s="15">
+        <v>8500</v>
+      </c>
+      <c r="D21" s="12">
+        <v>46314</v>
+      </c>
+      <c r="E21" s="11">
+        <v>70</v>
+      </c>
+      <c r="F21" s="11" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
-        <v>34</v>
+        <v>21</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C23" s="15">
+        <v>135161.25</v>
+      </c>
+      <c r="D23" s="12">
+        <v>46310</v>
+      </c>
+      <c r="E23" s="11">
+        <v>70</v>
+      </c>
+      <c r="F23" s="11" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
-        <v>35</v>
+        <v>32</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C24" s="15">
+        <v>1350000</v>
+      </c>
+      <c r="D24" s="12">
+        <v>46303</v>
+      </c>
+      <c r="E24" s="11">
+        <v>75</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B25" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="C25" s="16">
-        <v>6500</v>
-      </c>
-      <c r="D25" s="14">
-        <v>46308</v>
-      </c>
-      <c r="E25" s="13">
-        <v>75</v>
-      </c>
-      <c r="F25" s="13" t="s">
-        <v>71</v>
+        <v>22</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B26" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="C26" s="15">
-        <v>73000</v>
-      </c>
-      <c r="D26" s="12">
-        <v>46308</v>
-      </c>
-      <c r="E26" s="11">
-        <v>35</v>
-      </c>
-      <c r="F26" s="13" t="s">
-        <v>72</v>
+        <v>33</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B27" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="C27" s="15">
-        <v>450000</v>
-      </c>
-      <c r="D27" s="12">
-        <v>46309</v>
-      </c>
-      <c r="E27" s="11">
-        <v>50</v>
-      </c>
-      <c r="F27" s="13" t="s">
-        <v>81</v>
+        <v>34</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="s">
-        <v>40</v>
+        <v>36</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" s="16">
+        <v>6500</v>
+      </c>
+      <c r="D29" s="14">
+        <v>46308</v>
+      </c>
+      <c r="E29" s="13">
+        <v>75</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="C30" s="15">
-        <v>286200</v>
+        <v>73000</v>
       </c>
       <c r="D30" s="12">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="E30" s="11">
-        <v>100</v>
-      </c>
-      <c r="F30" s="11" t="s">
-        <v>69</v>
+        <v>35</v>
+      </c>
+      <c r="F30" s="13" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="11" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C31" s="15">
-        <v>16000</v>
+        <v>450000</v>
       </c>
       <c r="D31" s="12">
         <v>46309</v>
       </c>
       <c r="E31" s="11">
-        <v>70</v>
-      </c>
-      <c r="F31" s="11" t="s">
-        <v>76</v>
+        <v>50</v>
+      </c>
+      <c r="F31" s="13" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B32" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="C32" s="15">
-        <v>8000</v>
-      </c>
-      <c r="D32" s="12">
-        <v>46310</v>
-      </c>
-      <c r="E32" s="11">
-        <v>70</v>
-      </c>
-      <c r="F32" s="11" t="s">
-        <v>78</v>
+        <v>37</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B33" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="C33" s="15">
-        <v>80000</v>
-      </c>
-      <c r="D33" s="12">
-        <v>46310</v>
-      </c>
-      <c r="E33" s="11">
-        <v>100</v>
-      </c>
-      <c r="F33" s="11" t="s">
-        <v>80</v>
+        <v>40</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
@@ -1364,19 +1391,19 @@
         <v>41</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C34" s="15">
-        <v>1650</v>
+        <v>286200</v>
       </c>
       <c r="D34" s="12">
-        <v>46309</v>
+        <v>46304</v>
       </c>
       <c r="E34" s="11">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
@@ -1387,7 +1414,7 @@
         <v>61</v>
       </c>
       <c r="C35" s="15">
-        <v>8000</v>
+        <v>16000</v>
       </c>
       <c r="D35" s="12">
         <v>46309</v>
@@ -1396,46 +1423,126 @@
         <v>70</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
+      </c>
+      <c r="B36" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C36" s="15">
+        <v>8000</v>
+      </c>
+      <c r="D36" s="12">
+        <v>46310</v>
+      </c>
+      <c r="E36" s="11">
+        <v>70</v>
+      </c>
+      <c r="F36" s="11" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="11" t="s">
-        <v>43</v>
+        <v>41</v>
+      </c>
+      <c r="B37" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C37" s="15">
+        <v>80000</v>
+      </c>
+      <c r="D37" s="12">
+        <v>46310</v>
+      </c>
+      <c r="E37" s="11">
+        <v>100</v>
+      </c>
+      <c r="F37" s="11" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="11" t="s">
-        <v>44</v>
+        <v>41</v>
+      </c>
+      <c r="B38" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C38" s="15">
+        <v>1650</v>
+      </c>
+      <c r="D38" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E38" s="11">
+        <v>50</v>
+      </c>
+      <c r="F38" s="11" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="11" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C39" s="15">
-        <v>125000</v>
+        <v>8000</v>
       </c>
       <c r="D39" s="12">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="E39" s="11">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="11" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" s="11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B43" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C43" s="15">
+        <v>125000</v>
+      </c>
+      <c r="D43" s="12">
+        <v>46311</v>
+      </c>
+      <c r="E43" s="11">
+        <v>100</v>
+      </c>
+      <c r="F43" s="11" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" s="11" t="s">
         <v>46</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza painel (22/10/2026 15:09)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68E522AD-9860-4F6A-BD2D-39DA48FFFC2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{866EA0AC-D07B-488D-A33C-9941096295FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="96">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -332,6 +332,24 @@
   </si>
   <si>
     <t>690531126-48</t>
+  </si>
+  <si>
+    <t>690531038-123</t>
+  </si>
+  <si>
+    <t>690531094-37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Venda </t>
+  </si>
+  <si>
+    <t>690531114-14</t>
+  </si>
+  <si>
+    <t>690531104-972</t>
+  </si>
+  <si>
+    <t>690531104-973</t>
   </si>
 </sst>
 </file>
@@ -533,8 +551,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E69" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:E69" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E72" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:E72" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F68D7E3E-8D02-41D7-8907-35C934E19501}" name="Corretor" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{EACFDE5D-3403-4D4D-BD98-558F34E9A0F1}" name="Venda ou Locação" dataDxfId="5"/>
@@ -858,7 +876,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51DF420C-6417-4C8E-9CA8-EAE7781FF48D}">
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr defaultColWidth="26.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="26.44140625" style="11"/>
@@ -906,27 +924,42 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" s="15">
+        <v>240000</v>
+      </c>
+      <c r="D3" s="12">
+        <v>46315</v>
+      </c>
+      <c r="E3" s="11">
+        <v>130</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C4" s="15">
-        <v>185000</v>
+        <v>2200</v>
       </c>
       <c r="D4" s="12">
-        <v>46310</v>
+        <v>46316</v>
       </c>
       <c r="E4" s="11">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -934,99 +967,99 @@
         <v>25</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C5" s="15">
-        <v>1500</v>
+        <v>185000</v>
       </c>
       <c r="D5" s="12">
-        <v>46314</v>
+        <v>46310</v>
       </c>
       <c r="E5" s="11">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="C6" s="15">
-        <v>73000</v>
+        <v>1500</v>
       </c>
       <c r="D6" s="12">
-        <v>46308</v>
+        <v>46314</v>
       </c>
       <c r="E6" s="11">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="C7" s="15">
-        <v>1650</v>
+        <v>73000</v>
       </c>
       <c r="D7" s="12">
-        <v>46303</v>
+        <v>46308</v>
       </c>
       <c r="E7" s="11">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="C8" s="16">
-        <v>1350000</v>
-      </c>
-      <c r="D8" s="14">
+        <v>26</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="15">
+        <v>1650</v>
+      </c>
+      <c r="D8" s="12">
         <v>46303</v>
       </c>
-      <c r="E8" s="13">
-        <v>75</v>
-      </c>
-      <c r="F8" s="13" t="s">
-        <v>63</v>
+      <c r="E8" s="11">
+        <v>50</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="C9" s="15">
-        <v>100000</v>
-      </c>
-      <c r="D9" s="12">
-        <v>46308</v>
-      </c>
-      <c r="E9" s="11">
-        <v>100</v>
+      <c r="B9" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="C9" s="16">
+        <v>1350000</v>
+      </c>
+      <c r="D9" s="14">
+        <v>46303</v>
+      </c>
+      <c r="E9" s="13">
+        <v>75</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -1034,19 +1067,19 @@
         <v>27</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C10" s="15">
-        <v>450000</v>
+        <v>100000</v>
       </c>
       <c r="D10" s="12">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="E10" s="11">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -1054,99 +1087,99 @@
         <v>27</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C11" s="15">
-        <v>1700</v>
+        <v>450000</v>
       </c>
       <c r="D11" s="12">
-        <v>46315</v>
+        <v>46309</v>
       </c>
       <c r="E11" s="11">
         <v>50</v>
       </c>
       <c r="F11" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" s="15">
+        <v>1700</v>
+      </c>
+      <c r="D12" s="12">
+        <v>46315</v>
+      </c>
+      <c r="E12" s="11">
+        <v>50</v>
+      </c>
+      <c r="F12" s="13" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="C12" s="16">
-        <v>4400</v>
-      </c>
-      <c r="D12" s="14">
-        <v>46302</v>
-      </c>
-      <c r="E12" s="13">
-        <v>35</v>
-      </c>
-      <c r="F12" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
         <v>20</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C13" s="16">
-        <v>350000</v>
+        <v>4400</v>
       </c>
       <c r="D13" s="14">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E13" s="13">
-        <v>100</v>
+        <v>35</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B14" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="C14" s="15">
-        <v>320000</v>
-      </c>
-      <c r="D14" s="12">
-        <v>46309</v>
-      </c>
-      <c r="E14" s="11">
+      <c r="C14" s="16">
+        <v>350000</v>
+      </c>
+      <c r="D14" s="14">
+        <v>46303</v>
+      </c>
+      <c r="E14" s="13">
         <v>100</v>
       </c>
-      <c r="F14" s="11" t="s">
-        <v>73</v>
+      <c r="F14" s="13" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C15" s="15">
-        <v>2190</v>
+        <v>320000</v>
       </c>
       <c r="D15" s="12">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="E15" s="11">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>62</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -1154,41 +1187,44 @@
         <v>28</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C16" s="15">
-        <v>2100000</v>
+        <v>2190</v>
+      </c>
+      <c r="D16" s="12">
+        <v>46302</v>
       </c>
       <c r="E16" s="11">
-        <v>120</v>
+        <v>70</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>86</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C17" s="15">
+        <v>2100000</v>
+      </c>
+      <c r="D17" s="12">
+        <v>46312</v>
+      </c>
+      <c r="E17" s="11">
+        <v>120</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="C18" s="15">
-        <v>4400</v>
-      </c>
-      <c r="D18" s="12">
-        <v>46302</v>
-      </c>
-      <c r="E18" s="11">
-        <v>35</v>
-      </c>
-      <c r="F18" s="11" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -1196,19 +1232,19 @@
         <v>30</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="C19" s="15">
-        <v>2000</v>
+        <v>4400</v>
       </c>
       <c r="D19" s="12">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="E19" s="11">
+        <v>35</v>
+      </c>
+      <c r="F19" s="11" t="s">
         <v>50</v>
-      </c>
-      <c r="F19" s="11" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
@@ -1219,16 +1255,16 @@
         <v>61</v>
       </c>
       <c r="C20" s="15">
-        <v>2100</v>
+        <v>2000</v>
       </c>
       <c r="D20" s="12">
-        <v>46310</v>
+        <v>46304</v>
       </c>
       <c r="E20" s="11">
+        <v>50</v>
+      </c>
+      <c r="F20" s="11" t="s">
         <v>70</v>
-      </c>
-      <c r="F20" s="11" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -1239,211 +1275,226 @@
         <v>61</v>
       </c>
       <c r="C21" s="15">
-        <v>8500</v>
+        <v>2100</v>
       </c>
       <c r="D21" s="12">
-        <v>46314</v>
+        <v>46310</v>
       </c>
       <c r="E21" s="11">
         <v>70</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C22" s="15">
+        <v>8500</v>
+      </c>
+      <c r="D22" s="12">
+        <v>46314</v>
+      </c>
+      <c r="E22" s="11">
+        <v>70</v>
+      </c>
+      <c r="F22" s="11" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C23" s="15">
-        <v>135161.25</v>
+        <v>195000</v>
       </c>
       <c r="D23" s="12">
-        <v>46310</v>
+        <v>46316</v>
       </c>
       <c r="E23" s="11">
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C24" s="15">
-        <v>1350000</v>
+        <v>18000</v>
       </c>
       <c r="D24" s="12">
-        <v>46303</v>
+        <v>46316</v>
       </c>
       <c r="E24" s="11">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>63</v>
+        <v>95</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
-        <v>22</v>
+        <v>31</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C25" s="15">
+        <v>135000</v>
+      </c>
+      <c r="D25" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E25" s="11">
+        <v>130</v>
+      </c>
+      <c r="F25" s="11" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
-        <v>33</v>
+        <v>21</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C26" s="15">
+        <v>135161.25</v>
+      </c>
+      <c r="D26" s="12">
+        <v>46310</v>
+      </c>
+      <c r="E26" s="11">
+        <v>70</v>
+      </c>
+      <c r="F26" s="11" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="11" t="s">
-        <v>34</v>
+        <v>32</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C27" s="15">
+        <v>1350000</v>
+      </c>
+      <c r="D27" s="12">
+        <v>46303</v>
+      </c>
+      <c r="E27" s="11">
+        <v>75</v>
+      </c>
+      <c r="F27" s="11" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B29" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="C29" s="16">
-        <v>6500</v>
-      </c>
-      <c r="D29" s="14">
-        <v>46308</v>
-      </c>
-      <c r="E29" s="13">
-        <v>75</v>
-      </c>
-      <c r="F29" s="13" t="s">
-        <v>71</v>
+        <v>33</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B30" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="C30" s="15">
-        <v>73000</v>
-      </c>
-      <c r="D30" s="12">
-        <v>46308</v>
-      </c>
-      <c r="E30" s="11">
-        <v>35</v>
-      </c>
-      <c r="F30" s="13" t="s">
-        <v>72</v>
+        <v>34</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B31" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="C31" s="15">
-        <v>450000</v>
-      </c>
-      <c r="D31" s="12">
-        <v>46309</v>
-      </c>
-      <c r="E31" s="11">
-        <v>50</v>
-      </c>
-      <c r="F31" s="13" t="s">
-        <v>81</v>
+        <v>35</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
+      </c>
+      <c r="B32" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C32" s="16">
+        <v>6500</v>
+      </c>
+      <c r="D32" s="14">
+        <v>46308</v>
+      </c>
+      <c r="E32" s="13">
+        <v>75</v>
+      </c>
+      <c r="F32" s="13" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="11" t="s">
-        <v>40</v>
+        <v>36</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="C33" s="15">
+        <v>73000</v>
+      </c>
+      <c r="D33" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E33" s="11">
+        <v>35</v>
+      </c>
+      <c r="F33" s="13" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="11" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C34" s="15">
-        <v>286200</v>
+        <v>450000</v>
       </c>
       <c r="D34" s="12">
-        <v>46304</v>
+        <v>46309</v>
       </c>
       <c r="E34" s="11">
-        <v>100</v>
-      </c>
-      <c r="F34" s="11" t="s">
-        <v>69</v>
+        <v>50</v>
+      </c>
+      <c r="F34" s="13" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B35" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="C35" s="15">
-        <v>16000</v>
-      </c>
-      <c r="D35" s="12">
-        <v>46309</v>
-      </c>
-      <c r="E35" s="11">
-        <v>70</v>
-      </c>
-      <c r="F35" s="11" t="s">
-        <v>76</v>
+        <v>37</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B36" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="C36" s="15">
-        <v>8000</v>
-      </c>
-      <c r="D36" s="12">
-        <v>46310</v>
-      </c>
-      <c r="E36" s="11">
-        <v>70</v>
-      </c>
-      <c r="F36" s="11" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
@@ -1454,16 +1505,16 @@
         <v>66</v>
       </c>
       <c r="C37" s="15">
-        <v>80000</v>
+        <v>286200</v>
       </c>
       <c r="D37" s="12">
-        <v>46310</v>
+        <v>46304</v>
       </c>
       <c r="E37" s="11">
         <v>100</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
@@ -1474,16 +1525,16 @@
         <v>61</v>
       </c>
       <c r="C38" s="15">
-        <v>1650</v>
+        <v>16000</v>
       </c>
       <c r="D38" s="12">
         <v>46309</v>
       </c>
       <c r="E38" s="11">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
@@ -1497,52 +1548,112 @@
         <v>8000</v>
       </c>
       <c r="D39" s="12">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="E39" s="11">
         <v>70</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
+      </c>
+      <c r="B40" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C40" s="15">
+        <v>80000</v>
+      </c>
+      <c r="D40" s="12">
+        <v>46310</v>
+      </c>
+      <c r="E40" s="11">
+        <v>100</v>
+      </c>
+      <c r="F40" s="11" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="11" t="s">
-        <v>43</v>
+        <v>41</v>
+      </c>
+      <c r="B41" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C41" s="15">
+        <v>1650</v>
+      </c>
+      <c r="D41" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E41" s="11">
+        <v>50</v>
+      </c>
+      <c r="F41" s="11" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="11" t="s">
-        <v>44</v>
+        <v>41</v>
+      </c>
+      <c r="B42" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C42" s="15">
+        <v>8000</v>
+      </c>
+      <c r="D42" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E42" s="11">
+        <v>70</v>
+      </c>
+      <c r="F42" s="11" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="B43" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="C43" s="15">
-        <v>125000</v>
-      </c>
-      <c r="D43" s="12">
-        <v>46311</v>
-      </c>
-      <c r="E43" s="11">
-        <v>100</v>
-      </c>
-      <c r="F43" s="11" t="s">
-        <v>84</v>
+        <v>42</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" s="11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B46" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C46" s="15">
+        <v>125000</v>
+      </c>
+      <c r="D46" s="12">
+        <v>46311</v>
+      </c>
+      <c r="E46" s="11">
+        <v>100</v>
+      </c>
+      <c r="F46" s="11" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" s="11" t="s">
         <v>46</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza painel (23/10/2026 14:54)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{866EA0AC-D07B-488D-A33C-9941096295FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95A287A4-6EE9-49F9-AF3B-0908D1A26766}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="98">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -190,9 +190,6 @@
     <t>Fernanda Pacheco</t>
   </si>
   <si>
-    <t>Ademir Maia</t>
-  </si>
-  <si>
     <t>Gabriela Ferreira</t>
   </si>
   <si>
@@ -350,6 +347,15 @@
   </si>
   <si>
     <t>690531104-973</t>
+  </si>
+  <si>
+    <t>690531039-94</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Venda - Parceria </t>
+  </si>
+  <si>
+    <t>690531008-314</t>
   </si>
 </sst>
 </file>
@@ -551,8 +557,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E72" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:E72" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E74" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:E74" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F68D7E3E-8D02-41D7-8907-35C934E19501}" name="Corretor" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{EACFDE5D-3403-4D4D-BD98-558F34E9A0F1}" name="Venda ou Locação" dataDxfId="5"/>
@@ -876,7 +882,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51DF420C-6417-4C8E-9CA8-EAE7781FF48D}">
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr defaultColWidth="26.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="26.44140625" style="11"/>
@@ -890,13 +896,13 @@
         <v>15</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C1" s="15" t="s">
         <v>16</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E1" s="11" t="s">
         <v>17</v>
@@ -907,7 +913,7 @@
         <v>23</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C2" s="15">
         <v>2000</v>
@@ -919,7 +925,7 @@
         <v>50</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -927,7 +933,7 @@
         <v>23</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C3" s="15">
         <v>240000</v>
@@ -939,7 +945,7 @@
         <v>130</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -947,7 +953,7 @@
         <v>24</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C4" s="15">
         <v>2200</v>
@@ -959,7 +965,7 @@
         <v>70</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -967,7 +973,7 @@
         <v>25</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C5" s="15">
         <v>185000</v>
@@ -979,7 +985,7 @@
         <v>100</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -987,7 +993,7 @@
         <v>25</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C6" s="15">
         <v>1500</v>
@@ -999,7 +1005,7 @@
         <v>50</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -1007,7 +1013,7 @@
         <v>39</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C7" s="15">
         <v>73000</v>
@@ -1019,67 +1025,67 @@
         <v>35</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C8" s="15">
-        <v>1650</v>
+        <v>2400</v>
       </c>
       <c r="D8" s="12">
-        <v>46303</v>
+        <v>46317</v>
       </c>
       <c r="E8" s="11">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>65</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C9" s="15">
+        <v>1650</v>
+      </c>
+      <c r="D9" s="12">
+        <v>46303</v>
+      </c>
+      <c r="E9" s="11">
+        <v>50</v>
+      </c>
+      <c r="F9" s="11" t="s">
         <v>64</v>
-      </c>
-      <c r="C9" s="16">
-        <v>1350000</v>
-      </c>
-      <c r="D9" s="14">
-        <v>46303</v>
-      </c>
-      <c r="E9" s="13">
-        <v>75</v>
-      </c>
-      <c r="F9" s="13" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="C10" s="15">
-        <v>100000</v>
-      </c>
-      <c r="D10" s="12">
-        <v>46308</v>
-      </c>
-      <c r="E10" s="11">
-        <v>100</v>
+      <c r="B10" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" s="16">
+        <v>1350000</v>
+      </c>
+      <c r="D10" s="14">
+        <v>46303</v>
+      </c>
+      <c r="E10" s="13">
+        <v>75</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -1087,19 +1093,19 @@
         <v>27</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C11" s="15">
-        <v>450000</v>
+        <v>100000</v>
       </c>
       <c r="D11" s="12">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="E11" s="11">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -1107,164 +1113,164 @@
         <v>27</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C12" s="15">
-        <v>1700</v>
+        <v>450000</v>
       </c>
       <c r="D12" s="12">
-        <v>46315</v>
+        <v>46309</v>
       </c>
       <c r="E12" s="11">
         <v>50</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="C13" s="16">
-        <v>4400</v>
-      </c>
-      <c r="D13" s="14">
-        <v>46302</v>
-      </c>
-      <c r="E13" s="13">
-        <v>35</v>
+        <v>27</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C13" s="15">
+        <v>1700</v>
+      </c>
+      <c r="D13" s="12">
+        <v>46315</v>
+      </c>
+      <c r="E13" s="11">
+        <v>50</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>50</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="C14" s="15">
+        <v>380000</v>
+      </c>
+      <c r="D14" s="12">
+        <v>46318</v>
+      </c>
+      <c r="E14" s="11">
+        <v>50</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B15" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="C14" s="16">
-        <v>350000</v>
-      </c>
-      <c r="D14" s="14">
-        <v>46303</v>
-      </c>
-      <c r="E14" s="13">
-        <v>100</v>
-      </c>
-      <c r="F14" s="13" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="C15" s="15">
-        <v>320000</v>
-      </c>
-      <c r="D15" s="12">
-        <v>46309</v>
-      </c>
-      <c r="E15" s="11">
-        <v>100</v>
-      </c>
-      <c r="F15" s="11" t="s">
-        <v>73</v>
+      <c r="C15" s="16">
+        <v>4400</v>
+      </c>
+      <c r="D15" s="14">
+        <v>46302</v>
+      </c>
+      <c r="E15" s="13">
+        <v>35</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="C16" s="15">
-        <v>2190</v>
-      </c>
-      <c r="D16" s="12">
-        <v>46302</v>
-      </c>
-      <c r="E16" s="11">
-        <v>70</v>
-      </c>
-      <c r="F16" s="11" t="s">
-        <v>62</v>
+        <v>20</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C16" s="16">
+        <v>350000</v>
+      </c>
+      <c r="D16" s="14">
+        <v>46303</v>
+      </c>
+      <c r="E16" s="13">
+        <v>100</v>
+      </c>
+      <c r="F16" s="13" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C17" s="15">
-        <v>2100000</v>
+        <v>320000</v>
       </c>
       <c r="D17" s="12">
-        <v>46312</v>
+        <v>46309</v>
       </c>
       <c r="E17" s="11">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C18" s="15">
+        <v>2190</v>
+      </c>
+      <c r="D18" s="12">
+        <v>46302</v>
+      </c>
+      <c r="E18" s="11">
+        <v>70</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="C19" s="15">
-        <v>4400</v>
+        <v>2100000</v>
       </c>
       <c r="D19" s="12">
-        <v>46302</v>
+        <v>46312</v>
       </c>
       <c r="E19" s="11">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>50</v>
+        <v>85</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B20" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="C20" s="15">
-        <v>2000</v>
-      </c>
-      <c r="D20" s="12">
-        <v>46304</v>
-      </c>
-      <c r="E20" s="11">
-        <v>50</v>
-      </c>
-      <c r="F20" s="11" t="s">
-        <v>70</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -1272,19 +1278,19 @@
         <v>30</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="C21" s="15">
-        <v>2100</v>
+        <v>4400</v>
       </c>
       <c r="D21" s="12">
-        <v>46310</v>
+        <v>46302</v>
       </c>
       <c r="E21" s="11">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>82</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -1292,19 +1298,19 @@
         <v>30</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C22" s="15">
-        <v>8500</v>
+        <v>2000</v>
       </c>
       <c r="D22" s="12">
-        <v>46314</v>
+        <v>46304</v>
       </c>
       <c r="E22" s="11">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>85</v>
+        <v>69</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
@@ -1312,19 +1318,19 @@
         <v>30</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="C23" s="15">
-        <v>195000</v>
+        <v>2100</v>
       </c>
       <c r="D23" s="12">
-        <v>46316</v>
+        <v>46310</v>
       </c>
       <c r="E23" s="11">
-        <v>130</v>
+        <v>70</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>94</v>
+        <v>81</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -1332,33 +1338,33 @@
         <v>30</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C24" s="15">
-        <v>18000</v>
+        <v>8500</v>
       </c>
       <c r="D24" s="12">
-        <v>46316</v>
+        <v>46314</v>
       </c>
       <c r="E24" s="11">
         <v>70</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>92</v>
+        <v>65</v>
       </c>
       <c r="C25" s="15">
-        <v>135000</v>
+        <v>195000</v>
       </c>
       <c r="D25" s="12">
-        <v>46308</v>
+        <v>46316</v>
       </c>
       <c r="E25" s="11">
         <v>130</v>
@@ -1369,192 +1375,192 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C26" s="15">
-        <v>135161.25</v>
+        <v>18000</v>
       </c>
       <c r="D26" s="12">
-        <v>46310</v>
+        <v>46316</v>
       </c>
       <c r="E26" s="11">
         <v>70</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>64</v>
+        <v>91</v>
       </c>
       <c r="C27" s="15">
-        <v>1350000</v>
+        <v>135000</v>
       </c>
       <c r="D27" s="12">
-        <v>46303</v>
+        <v>46308</v>
       </c>
       <c r="E27" s="11">
-        <v>75</v>
+        <v>130</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>63</v>
+        <v>92</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C28" s="15">
+        <v>135161.25</v>
+      </c>
+      <c r="D28" s="12">
+        <v>46310</v>
+      </c>
+      <c r="E28" s="11">
+        <v>70</v>
+      </c>
+      <c r="F28" s="11" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
+      </c>
+      <c r="B29" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C29" s="15">
+        <v>1350000</v>
+      </c>
+      <c r="D29" s="12">
+        <v>46303</v>
+      </c>
+      <c r="E29" s="11">
+        <v>75</v>
+      </c>
+      <c r="F29" s="11" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
-        <v>34</v>
+        <v>32</v>
+      </c>
+      <c r="B30" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="C30" s="15">
+        <v>380000</v>
+      </c>
+      <c r="D30" s="12">
+        <v>46318</v>
+      </c>
+      <c r="E30" s="11">
+        <v>50</v>
+      </c>
+      <c r="F30" s="13" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="11" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B32" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="C32" s="16">
-        <v>6500</v>
-      </c>
-      <c r="D32" s="14">
-        <v>46308</v>
-      </c>
-      <c r="E32" s="13">
-        <v>75</v>
-      </c>
-      <c r="F32" s="13" t="s">
-        <v>71</v>
+        <v>33</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B33" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="C33" s="15">
-        <v>73000</v>
-      </c>
-      <c r="D33" s="12">
-        <v>46308</v>
-      </c>
-      <c r="E33" s="11">
-        <v>35</v>
-      </c>
-      <c r="F33" s="13" t="s">
-        <v>72</v>
+        <v>34</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B34" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="C34" s="15">
-        <v>450000</v>
-      </c>
-      <c r="D34" s="12">
-        <v>46309</v>
-      </c>
-      <c r="E34" s="11">
-        <v>50</v>
-      </c>
-      <c r="F34" s="13" t="s">
-        <v>81</v>
+        <v>35</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
+      </c>
+      <c r="B35" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="C35" s="16">
+        <v>6500</v>
+      </c>
+      <c r="D35" s="14">
+        <v>46308</v>
+      </c>
+      <c r="E35" s="13">
+        <v>75</v>
+      </c>
+      <c r="F35" s="13" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="11" t="s">
-        <v>40</v>
+        <v>36</v>
+      </c>
+      <c r="B36" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="C36" s="15">
+        <v>73000</v>
+      </c>
+      <c r="D36" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E36" s="11">
+        <v>35</v>
+      </c>
+      <c r="F36" s="13" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="11" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C37" s="15">
-        <v>286200</v>
+        <v>450000</v>
       </c>
       <c r="D37" s="12">
-        <v>46304</v>
+        <v>46309</v>
       </c>
       <c r="E37" s="11">
-        <v>100</v>
-      </c>
-      <c r="F37" s="11" t="s">
-        <v>69</v>
+        <v>50</v>
+      </c>
+      <c r="F37" s="13" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B38" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="C38" s="15">
-        <v>16000</v>
-      </c>
-      <c r="D38" s="12">
-        <v>46309</v>
-      </c>
-      <c r="E38" s="11">
-        <v>70</v>
-      </c>
-      <c r="F38" s="11" t="s">
-        <v>76</v>
+        <v>37</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B39" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="C39" s="15">
-        <v>8000</v>
-      </c>
-      <c r="D39" s="12">
-        <v>46310</v>
-      </c>
-      <c r="E39" s="11">
-        <v>70</v>
-      </c>
-      <c r="F39" s="11" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
@@ -1562,19 +1568,19 @@
         <v>41</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C40" s="15">
-        <v>80000</v>
+        <v>286200</v>
       </c>
       <c r="D40" s="12">
-        <v>46310</v>
+        <v>46304</v>
       </c>
       <c r="E40" s="11">
         <v>100</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
@@ -1582,19 +1588,19 @@
         <v>41</v>
       </c>
       <c r="B41" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C41" s="15">
-        <v>1650</v>
+        <v>16000</v>
       </c>
       <c r="D41" s="12">
         <v>46309</v>
       </c>
       <c r="E41" s="11">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
@@ -1602,13 +1608,13 @@
         <v>41</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C42" s="15">
         <v>8000</v>
       </c>
       <c r="D42" s="12">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="E42" s="11">
         <v>70</v>
@@ -1619,42 +1625,97 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
+      </c>
+      <c r="B43" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C43" s="15">
+        <v>80000</v>
+      </c>
+      <c r="D43" s="12">
+        <v>46310</v>
+      </c>
+      <c r="E43" s="11">
+        <v>100</v>
+      </c>
+      <c r="F43" s="11" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="11" t="s">
-        <v>43</v>
+        <v>41</v>
+      </c>
+      <c r="B44" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C44" s="15">
+        <v>1650</v>
+      </c>
+      <c r="D44" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E44" s="11">
+        <v>50</v>
+      </c>
+      <c r="F44" s="11" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="11" t="s">
-        <v>44</v>
+        <v>41</v>
+      </c>
+      <c r="B45" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C45" s="15">
+        <v>8000</v>
+      </c>
+      <c r="D45" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E45" s="11">
+        <v>70</v>
+      </c>
+      <c r="F45" s="11" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="B46" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="C46" s="15">
-        <v>125000</v>
-      </c>
-      <c r="D46" s="12">
-        <v>46311</v>
-      </c>
-      <c r="E46" s="11">
-        <v>100</v>
-      </c>
-      <c r="F46" s="11" t="s">
-        <v>84</v>
+        <v>42</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="11" t="s">
-        <v>46</v>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B48" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C48" s="15">
+        <v>125000</v>
+      </c>
+      <c r="D48" s="12">
+        <v>46311</v>
+      </c>
+      <c r="E48" s="11">
+        <v>100</v>
+      </c>
+      <c r="F48" s="11" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A49" s="11" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1699,7 +1760,7 @@
         <v>100</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -1709,7 +1770,7 @@
         <v>130</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -1719,7 +1780,7 @@
         <v>120</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -1729,7 +1790,7 @@
         <v>150</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -1739,7 +1800,7 @@
         <v>50</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -1749,7 +1810,7 @@
         <v>-50</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -1759,7 +1820,7 @@
         <v>200</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -1769,7 +1830,7 @@
         <v>50</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -1779,7 +1840,7 @@
         <v>70</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -1789,7 +1850,7 @@
         <v>-50</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualiza painel (23/10/2026 15:37)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95A287A4-6EE9-49F9-AF3B-0908D1A26766}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECC6022C-88D5-4885-B321-5D4459182583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="98">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -557,8 +557,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E74" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:E74" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E75" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:E75" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F68D7E3E-8D02-41D7-8907-35C934E19501}" name="Corretor" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{EACFDE5D-3403-4D4D-BD98-558F34E9A0F1}" name="Venda ou Locação" dataDxfId="5"/>
@@ -882,7 +882,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51DF420C-6417-4C8E-9CA8-EAE7781FF48D}">
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr defaultColWidth="26.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="26.44140625" style="11"/>
@@ -933,7 +933,7 @@
         <v>23</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C3" s="15">
         <v>240000</v>
@@ -942,7 +942,7 @@
         <v>46315</v>
       </c>
       <c r="E3" s="11">
-        <v>130</v>
+        <v>65</v>
       </c>
       <c r="F3" s="11" t="s">
         <v>90</v>
@@ -1395,62 +1395,62 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>91</v>
+        <v>63</v>
       </c>
       <c r="C27" s="15">
-        <v>135000</v>
+        <v>240000</v>
       </c>
       <c r="D27" s="12">
-        <v>46308</v>
+        <v>46315</v>
       </c>
       <c r="E27" s="11">
-        <v>130</v>
+        <v>65</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="C28" s="15">
-        <v>135161.25</v>
+        <v>135000</v>
       </c>
       <c r="D28" s="12">
-        <v>46310</v>
+        <v>46308</v>
       </c>
       <c r="E28" s="11">
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C29" s="15">
-        <v>1350000</v>
+        <v>135161.25</v>
       </c>
       <c r="D29" s="12">
-        <v>46303</v>
+        <v>46310</v>
       </c>
       <c r="E29" s="11">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>62</v>
+        <v>86</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
@@ -1458,79 +1458,79 @@
         <v>32</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>96</v>
+        <v>63</v>
       </c>
       <c r="C30" s="15">
-        <v>380000</v>
+        <v>1350000</v>
       </c>
       <c r="D30" s="12">
-        <v>46318</v>
+        <v>46303</v>
       </c>
       <c r="E30" s="11">
-        <v>50</v>
-      </c>
-      <c r="F30" s="13" t="s">
-        <v>97</v>
+        <v>75</v>
+      </c>
+      <c r="F30" s="11" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="11" t="s">
-        <v>22</v>
+        <v>32</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="C31" s="15">
+        <v>380000</v>
+      </c>
+      <c r="D31" s="12">
+        <v>46318</v>
+      </c>
+      <c r="E31" s="11">
+        <v>50</v>
+      </c>
+      <c r="F31" s="13" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B35" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="C35" s="16">
-        <v>6500</v>
-      </c>
-      <c r="D35" s="14">
-        <v>46308</v>
-      </c>
-      <c r="E35" s="13">
-        <v>75</v>
-      </c>
-      <c r="F35" s="13" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B36" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="C36" s="15">
-        <v>73000</v>
-      </c>
-      <c r="D36" s="12">
+      <c r="B36" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="C36" s="16">
+        <v>6500</v>
+      </c>
+      <c r="D36" s="14">
         <v>46308</v>
       </c>
-      <c r="E36" s="11">
-        <v>35</v>
+      <c r="E36" s="13">
+        <v>75</v>
       </c>
       <c r="F36" s="13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
@@ -1538,49 +1538,49 @@
         <v>36</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="C37" s="15">
-        <v>450000</v>
+        <v>73000</v>
       </c>
       <c r="D37" s="12">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="E37" s="11">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="F37" s="13" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
+      </c>
+      <c r="B38" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C38" s="15">
+        <v>450000</v>
+      </c>
+      <c r="D38" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E38" s="11">
+        <v>50</v>
+      </c>
+      <c r="F38" s="13" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B40" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="C40" s="15">
-        <v>286200</v>
-      </c>
-      <c r="D40" s="12">
-        <v>46304</v>
-      </c>
-      <c r="E40" s="11">
-        <v>100</v>
-      </c>
-      <c r="F40" s="11" t="s">
-        <v>68</v>
+        <v>40</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
@@ -1588,19 +1588,19 @@
         <v>41</v>
       </c>
       <c r="B41" s="11" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C41" s="15">
-        <v>16000</v>
+        <v>286200</v>
       </c>
       <c r="D41" s="12">
-        <v>46309</v>
+        <v>46304</v>
       </c>
       <c r="E41" s="11">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
@@ -1611,16 +1611,16 @@
         <v>60</v>
       </c>
       <c r="C42" s="15">
-        <v>8000</v>
+        <v>16000</v>
       </c>
       <c r="D42" s="12">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="E42" s="11">
         <v>70</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
@@ -1628,19 +1628,19 @@
         <v>41</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C43" s="15">
-        <v>80000</v>
+        <v>8000</v>
       </c>
       <c r="D43" s="12">
         <v>46310</v>
       </c>
       <c r="E43" s="11">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
@@ -1648,19 +1648,19 @@
         <v>41</v>
       </c>
       <c r="B44" s="11" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C44" s="15">
-        <v>1650</v>
+        <v>80000</v>
       </c>
       <c r="D44" s="12">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="E44" s="11">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
@@ -1671,50 +1671,70 @@
         <v>60</v>
       </c>
       <c r="C45" s="15">
-        <v>8000</v>
+        <v>1650</v>
       </c>
       <c r="D45" s="12">
         <v>46309</v>
       </c>
       <c r="E45" s="11">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
+      </c>
+      <c r="B46" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C46" s="15">
+        <v>8000</v>
+      </c>
+      <c r="D46" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E46" s="11">
+        <v>70</v>
+      </c>
+      <c r="F46" s="11" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="B48" s="11" t="s">
+      <c r="B49" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="C48" s="15">
+      <c r="C49" s="15">
         <v>125000</v>
       </c>
-      <c r="D48" s="12">
+      <c r="D49" s="12">
         <v>46311</v>
       </c>
-      <c r="E48" s="11">
+      <c r="E49" s="11">
         <v>100</v>
       </c>
-      <c r="F48" s="11" t="s">
+      <c r="F49" s="11" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A49" s="11" t="s">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A50" s="11" t="s">
         <v>45</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza painel (23/10/2026 15:51)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECC6022C-88D5-4885-B321-5D4459182583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E4DC598-5D05-4E68-9117-7E5A670876DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="100">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -356,6 +356,12 @@
   </si>
   <si>
     <t>690531008-314</t>
+  </si>
+  <si>
+    <t>690701045-2</t>
+  </si>
+  <si>
+    <t>690531082-91</t>
   </si>
 </sst>
 </file>
@@ -557,8 +563,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E75" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:E75" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E76" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:E76" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F68D7E3E-8D02-41D7-8907-35C934E19501}" name="Corretor" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{EACFDE5D-3403-4D4D-BD98-558F34E9A0F1}" name="Venda ou Locação" dataDxfId="5"/>
@@ -882,7 +888,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51DF420C-6417-4C8E-9CA8-EAE7781FF48D}">
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr defaultColWidth="26.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="26.44140625" style="11"/>
@@ -1122,7 +1128,7 @@
         <v>46309</v>
       </c>
       <c r="E12" s="11">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="F12" s="13" t="s">
         <v>80</v>
@@ -1497,6 +1503,21 @@
       <c r="A32" s="11" t="s">
         <v>22</v>
       </c>
+      <c r="B32" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C32" s="15">
+        <v>3500</v>
+      </c>
+      <c r="D32" s="12">
+        <v>46318</v>
+      </c>
+      <c r="E32" s="11">
+        <v>70</v>
+      </c>
+      <c r="F32" s="11" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="11" t="s">
@@ -1567,7 +1588,7 @@
         <v>46309</v>
       </c>
       <c r="E38" s="11">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="F38" s="13" t="s">
         <v>80</v>
@@ -1575,32 +1596,32 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
+      </c>
+      <c r="B39" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" s="15">
+        <v>196000</v>
+      </c>
+      <c r="D39" s="12">
+        <v>46318</v>
+      </c>
+      <c r="E39" s="11">
+        <v>130</v>
+      </c>
+      <c r="F39" s="13" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B41" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="C41" s="15">
-        <v>286200</v>
-      </c>
-      <c r="D41" s="12">
-        <v>46304</v>
-      </c>
-      <c r="E41" s="11">
-        <v>100</v>
-      </c>
-      <c r="F41" s="11" t="s">
-        <v>68</v>
+        <v>40</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
@@ -1608,19 +1629,19 @@
         <v>41</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C42" s="15">
-        <v>16000</v>
+        <v>286200</v>
       </c>
       <c r="D42" s="12">
-        <v>46309</v>
+        <v>46304</v>
       </c>
       <c r="E42" s="11">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
@@ -1631,16 +1652,16 @@
         <v>60</v>
       </c>
       <c r="C43" s="15">
-        <v>8000</v>
+        <v>16000</v>
       </c>
       <c r="D43" s="12">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="E43" s="11">
         <v>70</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
@@ -1648,19 +1669,19 @@
         <v>41</v>
       </c>
       <c r="B44" s="11" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C44" s="15">
-        <v>80000</v>
+        <v>8000</v>
       </c>
       <c r="D44" s="12">
         <v>46310</v>
       </c>
       <c r="E44" s="11">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
@@ -1668,19 +1689,19 @@
         <v>41</v>
       </c>
       <c r="B45" s="11" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C45" s="15">
-        <v>1650</v>
+        <v>80000</v>
       </c>
       <c r="D45" s="12">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="E45" s="11">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -1691,50 +1712,70 @@
         <v>60</v>
       </c>
       <c r="C46" s="15">
-        <v>8000</v>
+        <v>1650</v>
       </c>
       <c r="D46" s="12">
         <v>46309</v>
       </c>
       <c r="E46" s="11">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
+      </c>
+      <c r="B47" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C47" s="15">
+        <v>8000</v>
+      </c>
+      <c r="D47" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E47" s="11">
+        <v>70</v>
+      </c>
+      <c r="F47" s="11" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="B49" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="C49" s="15">
-        <v>125000</v>
-      </c>
-      <c r="D49" s="12">
-        <v>46311</v>
-      </c>
-      <c r="E49" s="11">
-        <v>100</v>
-      </c>
-      <c r="F49" s="11" t="s">
-        <v>83</v>
+        <v>43</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B50" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C50" s="15">
+        <v>125000</v>
+      </c>
+      <c r="D50" s="12">
+        <v>46311</v>
+      </c>
+      <c r="E50" s="11">
+        <v>100</v>
+      </c>
+      <c r="F50" s="11" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A51" s="11" t="s">
         <v>45</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza painel (23/10/2026 15:57)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E4DC598-5D05-4E68-9117-7E5A670876DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9582909F-6247-4374-99E9-3549DC9EA79A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="101">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -362,6 +362,9 @@
   </si>
   <si>
     <t>690531082-91</t>
+  </si>
+  <si>
+    <t>690701024-234</t>
   </si>
 </sst>
 </file>
@@ -563,8 +566,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E76" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:E76" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E77" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:E77" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F68D7E3E-8D02-41D7-8907-35C934E19501}" name="Corretor" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{EACFDE5D-3403-4D4D-BD98-558F34E9A0F1}" name="Venda ou Locação" dataDxfId="5"/>
@@ -888,7 +891,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51DF420C-6417-4C8E-9CA8-EAE7781FF48D}">
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr defaultColWidth="26.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="26.44140625" style="11"/>
@@ -1236,22 +1239,22 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="B18" s="11" t="s">
         <v>60</v>
       </c>
       <c r="C18" s="15">
-        <v>2190</v>
+        <v>3200</v>
       </c>
       <c r="D18" s="12">
-        <v>46302</v>
+        <v>46318</v>
       </c>
       <c r="E18" s="11">
         <v>70</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>61</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -1259,44 +1262,44 @@
         <v>28</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C19" s="15">
-        <v>2100000</v>
+        <v>2190</v>
       </c>
       <c r="D19" s="12">
-        <v>46312</v>
+        <v>46302</v>
       </c>
       <c r="E19" s="11">
-        <v>120</v>
+        <v>70</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>85</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C20" s="15">
+        <v>2100000</v>
+      </c>
+      <c r="D20" s="12">
+        <v>46312</v>
+      </c>
+      <c r="E20" s="11">
+        <v>120</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B21" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="C21" s="15">
-        <v>4400</v>
-      </c>
-      <c r="D21" s="12">
-        <v>46302</v>
-      </c>
-      <c r="E21" s="11">
-        <v>35</v>
-      </c>
-      <c r="F21" s="11" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -1304,19 +1307,19 @@
         <v>30</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="C22" s="15">
-        <v>2000</v>
+        <v>4400</v>
       </c>
       <c r="D22" s="12">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="E22" s="11">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>69</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
@@ -1327,16 +1330,16 @@
         <v>60</v>
       </c>
       <c r="C23" s="15">
-        <v>2100</v>
+        <v>2000</v>
       </c>
       <c r="D23" s="12">
-        <v>46310</v>
+        <v>46304</v>
       </c>
       <c r="E23" s="11">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -1347,16 +1350,16 @@
         <v>60</v>
       </c>
       <c r="C24" s="15">
-        <v>8500</v>
+        <v>2100</v>
       </c>
       <c r="D24" s="12">
-        <v>46314</v>
+        <v>46310</v>
       </c>
       <c r="E24" s="11">
         <v>70</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
@@ -1364,19 +1367,19 @@
         <v>30</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C25" s="15">
-        <v>195000</v>
+        <v>8500</v>
       </c>
       <c r="D25" s="12">
-        <v>46316</v>
+        <v>46314</v>
       </c>
       <c r="E25" s="11">
-        <v>130</v>
+        <v>70</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
@@ -1384,19 +1387,19 @@
         <v>30</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C26" s="15">
-        <v>18000</v>
+        <v>195000</v>
       </c>
       <c r="D26" s="12">
         <v>46316</v>
       </c>
       <c r="E26" s="11">
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
@@ -1404,79 +1407,79 @@
         <v>30</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C27" s="15">
-        <v>240000</v>
+        <v>18000</v>
       </c>
       <c r="D27" s="12">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="E27" s="11">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>91</v>
+        <v>63</v>
       </c>
       <c r="C28" s="15">
-        <v>135000</v>
+        <v>240000</v>
       </c>
       <c r="D28" s="12">
-        <v>46308</v>
+        <v>46315</v>
       </c>
       <c r="E28" s="11">
-        <v>130</v>
+        <v>65</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="C29" s="15">
-        <v>135161.25</v>
+        <v>135000</v>
       </c>
       <c r="D29" s="12">
-        <v>46310</v>
+        <v>46308</v>
       </c>
       <c r="E29" s="11">
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C30" s="15">
-        <v>1350000</v>
+        <v>135161.25</v>
       </c>
       <c r="D30" s="12">
-        <v>46303</v>
+        <v>46310</v>
       </c>
       <c r="E30" s="11">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>62</v>
+        <v>86</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
@@ -1484,94 +1487,94 @@
         <v>32</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>96</v>
+        <v>63</v>
       </c>
       <c r="C31" s="15">
-        <v>380000</v>
+        <v>1350000</v>
       </c>
       <c r="D31" s="12">
-        <v>46318</v>
+        <v>46303</v>
       </c>
       <c r="E31" s="11">
-        <v>50</v>
-      </c>
-      <c r="F31" s="13" t="s">
-        <v>97</v>
+        <v>75</v>
+      </c>
+      <c r="F31" s="11" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>60</v>
+        <v>96</v>
       </c>
       <c r="C32" s="15">
-        <v>3500</v>
+        <v>380000</v>
       </c>
       <c r="D32" s="12">
         <v>46318</v>
       </c>
       <c r="E32" s="11">
-        <v>70</v>
-      </c>
-      <c r="F32" s="11" t="s">
-        <v>98</v>
+        <v>50</v>
+      </c>
+      <c r="F32" s="13" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="11" t="s">
-        <v>33</v>
+        <v>22</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C33" s="15">
+        <v>3500</v>
+      </c>
+      <c r="D33" s="12">
+        <v>46318</v>
+      </c>
+      <c r="E33" s="11">
+        <v>70</v>
+      </c>
+      <c r="F33" s="11" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B36" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="C36" s="16">
-        <v>6500</v>
-      </c>
-      <c r="D36" s="14">
-        <v>46308</v>
-      </c>
-      <c r="E36" s="13">
-        <v>75</v>
-      </c>
-      <c r="F36" s="13" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B37" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="C37" s="15">
-        <v>73000</v>
-      </c>
-      <c r="D37" s="12">
+      <c r="B37" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="C37" s="16">
+        <v>6500</v>
+      </c>
+      <c r="D37" s="14">
         <v>46308</v>
       </c>
-      <c r="E37" s="11">
-        <v>35</v>
+      <c r="E37" s="13">
+        <v>75</v>
       </c>
       <c r="F37" s="13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
@@ -1579,19 +1582,19 @@
         <v>36</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="C38" s="15">
-        <v>450000</v>
+        <v>73000</v>
       </c>
       <c r="D38" s="12">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="E38" s="11">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="F38" s="13" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
@@ -1599,49 +1602,49 @@
         <v>36</v>
       </c>
       <c r="B39" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C39" s="15">
+        <v>450000</v>
+      </c>
+      <c r="D39" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E39" s="11">
         <v>65</v>
       </c>
-      <c r="C39" s="15">
-        <v>196000</v>
-      </c>
-      <c r="D39" s="12">
-        <v>46318</v>
-      </c>
-      <c r="E39" s="11">
-        <v>130</v>
-      </c>
       <c r="F39" s="13" t="s">
-        <v>99</v>
+        <v>80</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
+      </c>
+      <c r="B40" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C40" s="15">
+        <v>196000</v>
+      </c>
+      <c r="D40" s="12">
+        <v>46318</v>
+      </c>
+      <c r="E40" s="11">
+        <v>130</v>
+      </c>
+      <c r="F40" s="13" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B42" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="C42" s="15">
-        <v>286200</v>
-      </c>
-      <c r="D42" s="12">
-        <v>46304</v>
-      </c>
-      <c r="E42" s="11">
-        <v>100</v>
-      </c>
-      <c r="F42" s="11" t="s">
-        <v>68</v>
+        <v>40</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
@@ -1649,19 +1652,19 @@
         <v>41</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C43" s="15">
-        <v>16000</v>
+        <v>286200</v>
       </c>
       <c r="D43" s="12">
-        <v>46309</v>
+        <v>46304</v>
       </c>
       <c r="E43" s="11">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
@@ -1672,16 +1675,16 @@
         <v>60</v>
       </c>
       <c r="C44" s="15">
-        <v>8000</v>
+        <v>16000</v>
       </c>
       <c r="D44" s="12">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="E44" s="11">
         <v>70</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
@@ -1689,19 +1692,19 @@
         <v>41</v>
       </c>
       <c r="B45" s="11" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C45" s="15">
-        <v>80000</v>
+        <v>8000</v>
       </c>
       <c r="D45" s="12">
         <v>46310</v>
       </c>
       <c r="E45" s="11">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -1709,19 +1712,19 @@
         <v>41</v>
       </c>
       <c r="B46" s="11" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C46" s="15">
-        <v>1650</v>
+        <v>80000</v>
       </c>
       <c r="D46" s="12">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="E46" s="11">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
@@ -1732,50 +1735,70 @@
         <v>60</v>
       </c>
       <c r="C47" s="15">
-        <v>8000</v>
+        <v>1650</v>
       </c>
       <c r="D47" s="12">
         <v>46309</v>
       </c>
       <c r="E47" s="11">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="F47" s="11" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
+      </c>
+      <c r="B48" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C48" s="15">
+        <v>8000</v>
+      </c>
+      <c r="D48" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E48" s="11">
+        <v>70</v>
+      </c>
+      <c r="F48" s="11" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="B50" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="C50" s="15">
-        <v>125000</v>
-      </c>
-      <c r="D50" s="12">
-        <v>46311</v>
-      </c>
-      <c r="E50" s="11">
-        <v>100</v>
-      </c>
-      <c r="F50" s="11" t="s">
-        <v>83</v>
+        <v>43</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B51" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C51" s="15">
+        <v>125000</v>
+      </c>
+      <c r="D51" s="12">
+        <v>46311</v>
+      </c>
+      <c r="E51" s="11">
+        <v>100</v>
+      </c>
+      <c r="F51" s="11" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A52" s="11" t="s">
         <v>45</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza painel (29/10/2026 14:35)
</commit_message>
<xml_diff>
--- a/planilha.xlsx
+++ b/planilha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\ADMINISTRATIVO\CAMPANHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7856B138-AD9E-4903-90AC-14D7B9DFF208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28B07DDB-16D5-42E5-B60B-5B1F2E5DF351}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D0A569A-6401-4D69-B618-3CBD7EE2C304}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="113">
   <si>
     <t>Configuração da campanha</t>
   </si>
@@ -262,9 +262,6 @@
     <t>Venda</t>
   </si>
   <si>
-    <t>Locação  - Parceria</t>
-  </si>
-  <si>
     <t>690531057-138</t>
   </si>
   <si>
@@ -365,6 +362,45 @@
   </si>
   <si>
     <t>690701024-234</t>
+  </si>
+  <si>
+    <t>690701021-159</t>
+  </si>
+  <si>
+    <t>690531126-49</t>
+  </si>
+  <si>
+    <t>690531104-974</t>
+  </si>
+  <si>
+    <t>690531008-308</t>
+  </si>
+  <si>
+    <t>26/10/29026</t>
+  </si>
+  <si>
+    <t>690701039-14</t>
+  </si>
+  <si>
+    <t>690701039-13</t>
+  </si>
+  <si>
+    <t>690701021-160</t>
+  </si>
+  <si>
+    <t>690701021-161</t>
+  </si>
+  <si>
+    <t>690701024-235</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 690531094-38</t>
+  </si>
+  <si>
+    <t>690531094-40</t>
+  </si>
+  <si>
+    <t>690531094-39</t>
   </si>
 </sst>
 </file>
@@ -566,8 +602,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E77" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:E77" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}" name="tbCaptacoes" displayName="tbCaptacoes" ref="A1:E91" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:E91" xr:uid="{668B0985-EECF-492F-83D9-EA40CCED3F15}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F68D7E3E-8D02-41D7-8907-35C934E19501}" name="Corretor" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{EACFDE5D-3403-4D4D-BD98-558F34E9A0F1}" name="Venda ou Locação" dataDxfId="5"/>
@@ -891,7 +927,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51DF420C-6417-4C8E-9CA8-EAE7781FF48D}">
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F66"/>
   <sheetFormatPr defaultColWidth="26.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="26.44140625" style="11"/>
@@ -934,7 +970,7 @@
         <v>50</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -954,52 +990,52 @@
         <v>65</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B4" s="11" t="s">
         <v>60</v>
       </c>
       <c r="C4" s="15">
-        <v>2200</v>
+        <v>1800</v>
       </c>
       <c r="D4" s="12">
-        <v>46316</v>
+        <v>46323</v>
       </c>
       <c r="E4" s="11">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>89</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C5" s="15">
-        <v>185000</v>
+        <v>3500</v>
       </c>
       <c r="D5" s="12">
-        <v>46310</v>
+        <v>46323</v>
       </c>
       <c r="E5" s="11">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>82</v>
+        <v>111</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>60</v>
@@ -1008,418 +1044,418 @@
         <v>1500</v>
       </c>
       <c r="D6" s="12">
-        <v>46314</v>
+        <v>46323</v>
       </c>
       <c r="E6" s="11">
         <v>50</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>88</v>
+        <v>112</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="C7" s="15">
-        <v>73000</v>
+        <v>2200</v>
       </c>
       <c r="D7" s="12">
-        <v>46308</v>
+        <v>46316</v>
       </c>
       <c r="E7" s="11">
-        <v>35</v>
+        <v>70</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C8" s="15">
-        <v>2400</v>
+        <v>185000</v>
       </c>
       <c r="D8" s="12">
-        <v>46317</v>
+        <v>46310</v>
       </c>
       <c r="E8" s="11">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>60</v>
       </c>
       <c r="C9" s="15">
-        <v>1650</v>
+        <v>1500</v>
       </c>
       <c r="D9" s="12">
-        <v>46303</v>
+        <v>46314</v>
       </c>
       <c r="E9" s="11">
         <v>50</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>64</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="C10" s="16">
-        <v>1350000</v>
-      </c>
-      <c r="D10" s="14">
-        <v>46303</v>
-      </c>
-      <c r="E10" s="13">
-        <v>75</v>
-      </c>
-      <c r="F10" s="13" t="s">
-        <v>62</v>
+      <c r="C10" s="15">
+        <v>350000</v>
+      </c>
+      <c r="D10" s="12">
+        <v>46321</v>
+      </c>
+      <c r="E10" s="11">
+        <v>65</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="C11" s="15">
-        <v>100000</v>
+        <v>73000</v>
       </c>
       <c r="D11" s="12">
         <v>46308</v>
       </c>
       <c r="E11" s="11">
-        <v>100</v>
-      </c>
-      <c r="F11" s="13" t="s">
-        <v>74</v>
+        <v>35</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C12" s="15">
-        <v>450000</v>
+        <v>2400</v>
       </c>
       <c r="D12" s="12">
-        <v>46309</v>
+        <v>46317</v>
       </c>
       <c r="E12" s="11">
-        <v>65</v>
-      </c>
-      <c r="F12" s="13" t="s">
-        <v>80</v>
+        <v>70</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B13" s="11" t="s">
         <v>60</v>
       </c>
       <c r="C13" s="15">
-        <v>1700</v>
+        <v>1650</v>
       </c>
       <c r="D13" s="12">
-        <v>46315</v>
+        <v>46303</v>
       </c>
       <c r="E13" s="11">
         <v>50</v>
       </c>
-      <c r="F13" s="13" t="s">
-        <v>87</v>
+      <c r="F13" s="11" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="C14" s="15">
-        <v>380000</v>
-      </c>
-      <c r="D14" s="12">
-        <v>46318</v>
-      </c>
-      <c r="E14" s="11">
-        <v>50</v>
+      <c r="B14" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="C14" s="16">
+        <v>1350000</v>
+      </c>
+      <c r="D14" s="14">
+        <v>46303</v>
+      </c>
+      <c r="E14" s="13">
+        <v>75</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="C15" s="16">
-        <v>4400</v>
-      </c>
-      <c r="D15" s="14">
-        <v>46302</v>
-      </c>
-      <c r="E15" s="13">
-        <v>35</v>
+        <v>27</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C15" s="15">
+        <v>100000</v>
+      </c>
+      <c r="D15" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E15" s="11">
+        <v>100</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>49</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C16" s="15">
+        <v>450000</v>
+      </c>
+      <c r="D16" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E16" s="11">
         <v>65</v>
       </c>
-      <c r="C16" s="16">
-        <v>350000</v>
-      </c>
-      <c r="D16" s="14">
-        <v>46303</v>
-      </c>
-      <c r="E16" s="13">
-        <v>100</v>
-      </c>
       <c r="F16" s="13" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C17" s="15">
-        <v>320000</v>
+        <v>1700</v>
       </c>
       <c r="D17" s="12">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="E17" s="11">
-        <v>100</v>
-      </c>
-      <c r="F17" s="11" t="s">
-        <v>72</v>
+        <v>50</v>
+      </c>
+      <c r="F17" s="13" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>60</v>
+        <v>95</v>
       </c>
       <c r="C18" s="15">
-        <v>3200</v>
+        <v>380000</v>
       </c>
       <c r="D18" s="12">
         <v>46318</v>
       </c>
       <c r="E18" s="11">
-        <v>70</v>
-      </c>
-      <c r="F18" s="11" t="s">
-        <v>100</v>
+        <v>50</v>
+      </c>
+      <c r="F18" s="13" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C19" s="15">
-        <v>2190</v>
+        <v>530000</v>
       </c>
       <c r="D19" s="12">
+        <v>46321</v>
+      </c>
+      <c r="E19" s="11">
+        <v>150</v>
+      </c>
+      <c r="F19" s="13" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="C20" s="16">
+        <v>4400</v>
+      </c>
+      <c r="D20" s="14">
         <v>46302</v>
       </c>
-      <c r="E19" s="11">
-        <v>70</v>
-      </c>
-      <c r="F19" s="11" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="B20" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="C20" s="15">
-        <v>2100000</v>
-      </c>
-      <c r="D20" s="12">
-        <v>46312</v>
-      </c>
-      <c r="E20" s="11">
-        <v>120</v>
-      </c>
-      <c r="F20" s="11" t="s">
-        <v>85</v>
+      <c r="E20" s="13">
+        <v>35</v>
+      </c>
+      <c r="F20" s="13" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
-        <v>29</v>
+        <v>20</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C21" s="16">
+        <v>350000</v>
+      </c>
+      <c r="D21" s="14">
+        <v>46303</v>
+      </c>
+      <c r="E21" s="13">
+        <v>100</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="C22" s="15">
-        <v>4400</v>
+        <v>320000</v>
       </c>
       <c r="D22" s="12">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="E22" s="11">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>49</v>
+        <v>71</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="B23" s="11" t="s">
         <v>60</v>
       </c>
       <c r="C23" s="15">
-        <v>2000</v>
+        <v>3200</v>
       </c>
       <c r="D23" s="12">
-        <v>46304</v>
+        <v>46318</v>
       </c>
       <c r="E23" s="11">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>69</v>
+        <v>99</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="B24" s="11" t="s">
         <v>60</v>
       </c>
       <c r="C24" s="15">
-        <v>2100</v>
+        <v>25000</v>
       </c>
       <c r="D24" s="12">
-        <v>46310</v>
+        <v>46353</v>
       </c>
       <c r="E24" s="11">
         <v>70</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>81</v>
+        <v>109</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B25" s="11" t="s">
         <v>60</v>
       </c>
       <c r="C25" s="15">
-        <v>8500</v>
+        <v>2190</v>
       </c>
       <c r="D25" s="12">
-        <v>46314</v>
+        <v>46302</v>
       </c>
       <c r="E25" s="11">
         <v>70</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>84</v>
+        <v>61</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B26" s="11" t="s">
         <v>65</v>
       </c>
       <c r="C26" s="15">
-        <v>195000</v>
+        <v>2100000</v>
       </c>
       <c r="D26" s="12">
-        <v>46316</v>
+        <v>46312</v>
       </c>
       <c r="E26" s="11">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B27" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="C27" s="15">
-        <v>18000</v>
-      </c>
-      <c r="D27" s="12">
-        <v>46316</v>
-      </c>
-      <c r="E27" s="11">
-        <v>70</v>
-      </c>
-      <c r="F27" s="11" t="s">
-        <v>94</v>
+        <v>29</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
@@ -1427,50 +1463,50 @@
         <v>30</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="C28" s="15">
-        <v>240000</v>
+        <v>4400</v>
       </c>
       <c r="D28" s="12">
-        <v>46315</v>
+        <v>46302</v>
       </c>
       <c r="E28" s="11">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>90</v>
+        <v>49</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>91</v>
+        <v>60</v>
       </c>
       <c r="C29" s="15">
-        <v>135000</v>
+        <v>2000</v>
       </c>
       <c r="D29" s="12">
-        <v>46308</v>
+        <v>46304</v>
       </c>
       <c r="E29" s="11">
-        <v>130</v>
+        <v>50</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>92</v>
+        <v>68</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="B30" s="11" t="s">
         <v>60</v>
       </c>
       <c r="C30" s="15">
-        <v>135161.25</v>
+        <v>2100</v>
       </c>
       <c r="D30" s="12">
         <v>46310</v>
@@ -1479,326 +1515,606 @@
         <v>70</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="11" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C31" s="15">
-        <v>1350000</v>
+        <v>8500</v>
       </c>
       <c r="D31" s="12">
-        <v>46303</v>
+        <v>46314</v>
       </c>
       <c r="E31" s="11">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>62</v>
+        <v>83</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="C32" s="15">
-        <v>380000</v>
+        <v>195000</v>
       </c>
       <c r="D32" s="12">
-        <v>46318</v>
+        <v>46316</v>
       </c>
       <c r="E32" s="11">
-        <v>50</v>
-      </c>
-      <c r="F32" s="13" t="s">
-        <v>97</v>
+        <v>130</v>
+      </c>
+      <c r="F32" s="11" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="11" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="B33" s="11" t="s">
         <v>60</v>
       </c>
       <c r="C33" s="15">
-        <v>3500</v>
+        <v>18000</v>
       </c>
       <c r="D33" s="12">
-        <v>46318</v>
+        <v>46316</v>
       </c>
       <c r="E33" s="11">
         <v>70</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
+      </c>
+      <c r="B34" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C34" s="15">
+        <v>240000</v>
+      </c>
+      <c r="D34" s="12">
+        <v>46315</v>
+      </c>
+      <c r="E34" s="11">
+        <v>65</v>
+      </c>
+      <c r="F34" s="11" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="11" t="s">
-        <v>34</v>
+        <v>30</v>
+      </c>
+      <c r="B35" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C35" s="15">
+        <v>350000</v>
+      </c>
+      <c r="D35" s="12">
+        <v>46321</v>
+      </c>
+      <c r="E35" s="11">
+        <v>65</v>
+      </c>
+      <c r="F35" s="11" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="11" t="s">
-        <v>35</v>
+        <v>30</v>
+      </c>
+      <c r="B36" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C36" s="15">
+        <v>4500</v>
+      </c>
+      <c r="D36" s="12">
+        <v>46322</v>
+      </c>
+      <c r="E36" s="11">
+        <v>70</v>
+      </c>
+      <c r="F36" s="11" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B37" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="C37" s="16">
-        <v>6500</v>
-      </c>
-      <c r="D37" s="14">
+        <v>31</v>
+      </c>
+      <c r="B37" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="C37" s="15">
+        <v>135000</v>
+      </c>
+      <c r="D37" s="12">
         <v>46308</v>
       </c>
-      <c r="E37" s="13">
-        <v>75</v>
-      </c>
-      <c r="F37" s="13" t="s">
-        <v>70</v>
+      <c r="E37" s="11">
+        <v>130</v>
+      </c>
+      <c r="F37" s="11" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="11" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="C38" s="15">
-        <v>73000</v>
+        <v>135161.25</v>
       </c>
       <c r="D38" s="12">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="E38" s="11">
-        <v>35</v>
-      </c>
-      <c r="F38" s="13" t="s">
-        <v>71</v>
+        <v>70</v>
+      </c>
+      <c r="F38" s="11" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="11" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C39" s="15">
-        <v>450000</v>
+        <v>1600</v>
       </c>
       <c r="D39" s="12">
-        <v>46309</v>
+        <v>46318</v>
       </c>
       <c r="E39" s="11">
-        <v>65</v>
-      </c>
-      <c r="F39" s="13" t="s">
-        <v>80</v>
+        <v>50</v>
+      </c>
+      <c r="F39" s="11" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="11" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="B40" s="11" t="s">
         <v>65</v>
       </c>
       <c r="C40" s="15">
-        <v>196000</v>
+        <v>320000</v>
       </c>
       <c r="D40" s="12">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="E40" s="11">
         <v>130</v>
       </c>
-      <c r="F40" s="13" t="s">
-        <v>99</v>
+      <c r="F40" s="11" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="11" t="s">
-        <v>37</v>
+        <v>21</v>
+      </c>
+      <c r="B41" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C41" s="15">
+        <v>790000</v>
+      </c>
+      <c r="D41" s="12">
+        <v>46322</v>
+      </c>
+      <c r="E41" s="11">
+        <v>150</v>
+      </c>
+      <c r="F41" s="11" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="11" t="s">
-        <v>40</v>
+        <v>32</v>
+      </c>
+      <c r="B42" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C42" s="15">
+        <v>1350000</v>
+      </c>
+      <c r="D42" s="12">
+        <v>46303</v>
+      </c>
+      <c r="E42" s="11">
+        <v>75</v>
+      </c>
+      <c r="F42" s="11" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="11" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>65</v>
+        <v>95</v>
       </c>
       <c r="C43" s="15">
-        <v>286200</v>
+        <v>380000</v>
       </c>
       <c r="D43" s="12">
-        <v>46304</v>
+        <v>46318</v>
       </c>
       <c r="E43" s="11">
-        <v>100</v>
-      </c>
-      <c r="F43" s="11" t="s">
-        <v>68</v>
+        <v>50</v>
+      </c>
+      <c r="F43" s="13" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="11" t="s">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="B44" s="11" t="s">
         <v>60</v>
       </c>
       <c r="C44" s="15">
-        <v>16000</v>
+        <v>3500</v>
       </c>
       <c r="D44" s="12">
-        <v>46309</v>
+        <v>46318</v>
       </c>
       <c r="E44" s="11">
         <v>70</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>75</v>
+        <v>97</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="11" t="s">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="B45" s="11" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="C45" s="15">
-        <v>8000</v>
+        <v>3200</v>
       </c>
       <c r="D45" s="12">
-        <v>46310</v>
+        <v>46321</v>
       </c>
       <c r="E45" s="11">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>77</v>
+        <v>106</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B46" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="C46" s="15">
-        <v>80000</v>
-      </c>
-      <c r="D46" s="12">
-        <v>46310</v>
-      </c>
-      <c r="E46" s="11">
-        <v>100</v>
-      </c>
-      <c r="F46" s="11" t="s">
-        <v>79</v>
+        <v>33</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B47" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="C47" s="15">
-        <v>1650</v>
-      </c>
-      <c r="D47" s="12">
-        <v>46309</v>
-      </c>
-      <c r="E47" s="11">
-        <v>50</v>
-      </c>
-      <c r="F47" s="11" t="s">
-        <v>78</v>
+        <v>34</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B48" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="C48" s="15">
-        <v>8000</v>
-      </c>
-      <c r="D48" s="12">
-        <v>46309</v>
-      </c>
-      <c r="E48" s="11">
-        <v>70</v>
-      </c>
-      <c r="F48" s="11" t="s">
-        <v>76</v>
+        <v>35</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="11" t="s">
-        <v>42</v>
+        <v>36</v>
+      </c>
+      <c r="B49" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="C49" s="16">
+        <v>6500</v>
+      </c>
+      <c r="D49" s="14">
+        <v>46308</v>
+      </c>
+      <c r="E49" s="13">
+        <v>75</v>
+      </c>
+      <c r="F49" s="13" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="11" t="s">
-        <v>43</v>
+        <v>36</v>
+      </c>
+      <c r="B50" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="C50" s="15">
+        <v>73000</v>
+      </c>
+      <c r="D50" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E50" s="11">
+        <v>35</v>
+      </c>
+      <c r="F50" s="13" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="11" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="B51" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C51" s="15">
+        <v>450000</v>
+      </c>
+      <c r="D51" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E51" s="11">
         <v>65</v>
       </c>
-      <c r="C51" s="15">
-        <v>125000</v>
-      </c>
-      <c r="D51" s="12">
-        <v>46311</v>
-      </c>
-      <c r="E51" s="11">
-        <v>100</v>
-      </c>
-      <c r="F51" s="11" t="s">
-        <v>83</v>
+      <c r="F51" s="13" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B52" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C52" s="15">
+        <v>196000</v>
+      </c>
+      <c r="D52" s="12">
+        <v>46318</v>
+      </c>
+      <c r="E52" s="11">
+        <v>130</v>
+      </c>
+      <c r="F52" s="13" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A53" s="11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A54" s="11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A55" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B55" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C55" s="15">
+        <v>286200</v>
+      </c>
+      <c r="D55" s="12">
+        <v>46304</v>
+      </c>
+      <c r="E55" s="11">
+        <v>100</v>
+      </c>
+      <c r="F55" s="11" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A56" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B56" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C56" s="15">
+        <v>16000</v>
+      </c>
+      <c r="D56" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E56" s="11">
+        <v>70</v>
+      </c>
+      <c r="F56" s="11" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A57" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B57" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C57" s="15">
+        <v>8000</v>
+      </c>
+      <c r="D57" s="12">
+        <v>46310</v>
+      </c>
+      <c r="E57" s="11">
+        <v>70</v>
+      </c>
+      <c r="F57" s="11" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A58" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B58" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C58" s="15">
+        <v>80000</v>
+      </c>
+      <c r="D58" s="12">
+        <v>46310</v>
+      </c>
+      <c r="E58" s="11">
+        <v>100</v>
+      </c>
+      <c r="F58" s="11" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A59" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B59" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C59" s="15">
+        <v>1650</v>
+      </c>
+      <c r="D59" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E59" s="11">
+        <v>50</v>
+      </c>
+      <c r="F59" s="11" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A60" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B60" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C60" s="15">
+        <v>8000</v>
+      </c>
+      <c r="D60" s="12">
+        <v>46309</v>
+      </c>
+      <c r="E60" s="11">
+        <v>70</v>
+      </c>
+      <c r="F60" s="11" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A61" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B61" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C61" s="15">
+        <v>1400</v>
+      </c>
+      <c r="D61" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="E61" s="11">
+        <v>50</v>
+      </c>
+      <c r="F61" s="11" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A62" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B62" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="C62" s="15">
+        <v>3200</v>
+      </c>
+      <c r="D62" s="12">
+        <v>46321</v>
+      </c>
+      <c r="E62" s="11">
+        <v>35</v>
+      </c>
+      <c r="F62" s="11" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A63" s="11" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A64" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A65" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B65" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C65" s="15">
+        <v>125000</v>
+      </c>
+      <c r="D65" s="12">
+        <v>46311</v>
+      </c>
+      <c r="E65" s="11">
+        <v>100</v>
+      </c>
+      <c r="F65" s="11" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A66" s="11" t="s">
         <v>45</v>
       </c>
     </row>

</xml_diff>